<commit_message>
replace k2 with agent loop
</commit_message>
<xml_diff>
--- a/backend/sample_markets_ml.xlsx
+++ b/backend/sample_markets_ml.xlsx
@@ -657,7 +657,7 @@
         <v>45827.76641976263</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>46110.07607241747</v>
+        <v>46110.28024383638</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>46109.32077546296</v>
@@ -703,10 +703,10 @@
         <v>25350912.14729484</v>
       </c>
       <c r="AB2" t="n">
-        <v>1411060.860000005</v>
+        <v>1352271.967000002</v>
       </c>
       <c r="AC2" t="n">
-        <v>5104747.474501974</v>
+        <v>5070154.290501975</v>
       </c>
       <c r="AD2" t="n">
         <v>25350912.1472949</v>
@@ -729,14 +729,14 @@
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>{"id": "553878", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/nba-finals-points-leader-7g2ZEZvMXxLb.jpg", "slug": "will-the-chicago-bulls-win-the-2026-nba-finals", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/nba-finals-points-leader-7g2ZEZvMXxLb.jpg", "ready": false, "active": true, "closed": true, "events": [{"id": "27830", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/nba-finals-points-leader-7g2ZEZvMXxLb.jpg", "slug": "2026-nba-champion", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/nba-finals-points-leader-7g2ZEZvMXxLb.jpg", "title": "2026 NBA Champion", "active": true, "closed": false, "sortBy": "price", "ticker": "2026-nba-champion", "volume": 207394956.867415, "endDate": "2026-07-01T00:00:00Z", "negRisk": true, "archived": false, "featured": false, "createdAt": "2025-06-19T18:23:26.785626Z", "deploying": false, "liquidity": 10039428.92563, "startDate": "2025-06-23T16:04:37.82012Z", "updatedAt": "2026-03-29T01:49:32.895725Z", "volume1mo": 73091497.38166507, "volume1wk": 17785304.81427103, "volume1yr": 207394956.86741585, "restricted": true, "volume24hr": 2335162.860974, "competitive": 0.9846153846153846, "description": "This market is to predict the winner of the 2025–26 NBA Finals.", "commentCount": 259, "creationDate": "2025-06-23T16:04:37.820118Z", "gmpChartMode": "default", "openInterest": 2706230.92922, "enableNegRisk": true, "eventMetadata": {"context_updated_at": "2026-03-29T01:46:27.538Z", "context_description": "Oklahoma City Thunder lead Polymarket's 2026 NBA Champion market at 37.5% implied probability, reflecting their league-best 57-16 record and first-to-clinch playoff berth in the stacked Western Conference, bolstered by Shai Gilgeous-Alexander's MVP-caliber play and a dominant 131-113 win over Chicago on March 27 featuring a 22-0 second-half run. San Antonio Spurs trail at 15.6% amid a scorching seven-game win streak—including a 123-98 rout of Memphis on March 25—fueled by Victor Wembanyama's MVP candidacy and the NBA's deepest roster, closing the gap on OKC in standings (55-18). Boston Celtics hold third at 11.5% with a solid 49-24 East mark, though Detroit Pistons' surge (53-20) intensifies conference finals path; Denver Nuggets (8.5%) rely on Nikola Jokić's historic triple-doubles despite middling 46-28 standing. Trader consensus prices emphasize West dominance, health, and late-season momentum with under 10 games left.", "context_requires_regen": true}, "liquidityClob": 10039428.92563, "enableOrderBook": true, "negRiskMarketID": "0x11e9a09023ace3097de216497c6fc01a57a57d63df7370543f288b40251dda00", "showAllOutcomes": true, "negRiskAugmented": false, "resolutionSource": "", "showMarketImages": false, "cumulativeMarkets": false, "pendingDeployment": false, "deployingTimestamp": "2025-06-23T15:28:44.417702Z", "automaticallyActive": true, "requiresTranslation": false}], "funded": false, "spread": 0.001, "volume": "25350912.14729484", "bestAsk": 0.001, "endDate": "2026-07-01T00:00:00Z", "feeType": null, "negRisk": true, "umaBond": "500", "approved": true, "archived": false, "featured": false, "outcomes": "[\"Yes\", \"No\"]", "question": "Will the Chicago Bulls win the 2026 NBA Finals?", "createdAt": "2025-06-19T18:23:38.667491Z", "deploying": false, "startDate": "2025-06-23T16:02:42.983826Z", "umaReward": "5", "updatedAt": "2026-03-29T01:49:32.656869Z", "volume1mo": 5104747.474501974, "volume1wk": 1411060.8600000052, "volume1yr": 25350912.147294898, "volumeNum": 25350912.14729484, "closedTime": "2026-03-28 07:41:55+00", "endDateIso": "2026-07-01", "questionID": "0x11e9a09023ace3097de216497c6fc01a57a57d63df7370543f288b40251dda16", "resolvedBy": "0x2F5e3684cb1F318ec51b00Edba38d79Ac2c0aA9d", "restricted": true, "rfqEnabled": false, "umaEndDate": "2026-03-28T07:41:55Z", "volume24hr": 1495.73, "volumeClob": 25350912.14729484, "conditionId": "0xf374fb58698bccedf29399f9f5548a70370a11c0fece34f2570fb9b3885e8e5a", "description": "This market will resolve to “Yes” if the Chicago Bulls win the 2026 NBA Finals. Otherwise, this market will resolve to “No”.\n\nThis market will resolve to “No” if it becomes impossible for this team to win the 2026 NBA Finals based off the rules of the NBA.\n\nThe resolution source for this market will be information from the NBA.", "feesEnabled": false, "seriesColor": "", "clobTokenIds": "[\"101657448900324364213467059356648689270832606863187352286785694887095023173679\", \"95109892472860043698165831230345254090456546311265426162114533642591273071363\"]", "negRiskOther": false, "orderMinSize": 5, "startDateIso": "2025-06-23", "submitted_by": "0x91430CaD2d3975766499717fA0D66A78D814E5c5", "outcomePrices": "[\"0\", \"1\"]", "showGmpSeries": false, "volume1moClob": 5104747.474501974, "volume1wkClob": 1411060.8600000052, "volume1yrClob": 25350912.147294898, "groupItemTitle": "Chicago Bulls", "lastTradePrice": 0.001, "rewardsMinSize": 20, "showGmpOutcome": false, "volume24hrClob": 1495.73, "acceptingOrders": false, "enableOrderBook": true, "negRiskMarketID": "0x11e9a09023ace3097de216497c6fc01a57a57d63df7370543f288b40251dda00", "clearBookOnStart": true, "hasReviewedDates": true, "manualActivation": false, "negRiskRequestID": "0x44221a0b742694c3114c7c93af03ea33e6ac61fa9e4854a019301ff03ff2f447", "resolutionSource": "", "rewardsMaxSpread": 3.5, "pendingDeployment": false, "deployingTimestamp": "2025-06-23T15:35:36.478958Z", "groupItemThreshold": "22", "marketMakerAddress": "", "automaticallyActive": true, "oneMonthPriceChange": -0.002, "requiresTranslation": false, "umaResolutionStatus": "resolved", "automaticallyResolved": true, "holdingRewardsEnabled": false, "orderPriceMinTickSize": 0.001, "umaResolutionStatuses": "[\"proposed\", \"resolved\"]", "acceptingOrdersTimestamp": "2025-06-23T16:02:15Z", "pagerDutyNotificationEnabled": false}</t>
+          <t>{"id": "553878", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/nba-finals-points-leader-7g2ZEZvMXxLb.jpg", "slug": "will-the-chicago-bulls-win-the-2026-nba-finals", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/nba-finals-points-leader-7g2ZEZvMXxLb.jpg", "ready": false, "active": true, "closed": true, "events": [{"id": "27830", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/nba-finals-points-leader-7g2ZEZvMXxLb.jpg", "slug": "2026-nba-champion", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/nba-finals-points-leader-7g2ZEZvMXxLb.jpg", "title": "2026 NBA Champion", "active": true, "closed": false, "sortBy": "price", "ticker": "2026-nba-champion", "volume": 207959072.18360305, "endDate": "2026-07-01T00:00:00Z", "negRisk": true, "archived": false, "featured": false, "createdAt": "2025-06-19T18:23:26.785626Z", "deploying": false, "liquidity": 8098580.77391, "startDate": "2025-06-23T16:04:37.82012Z", "updatedAt": "2026-03-29T06:43:33.736055Z", "volume1mo": 72985303.69146004, "volume1wk": 17899490.499662023, "volume1yr": 207959072.18360385, "restricted": true, "volume24hr": 2322731.1560189994, "competitive": 0.9846153846153846, "description": "This market is to predict the winner of the 2025–26 NBA Finals.", "commentCount": 260, "creationDate": "2025-06-23T16:04:37.820118Z", "gmpChartMode": "default", "openInterest": 2787127.0686719995, "enableNegRisk": true, "eventMetadata": {"context_updated_at": "2026-03-29T06:30:50.883Z", "context_description": "Oklahoma City Thunder command 37.5% implied probability as 2026 NBA champions per trader consensus, fueled by their NBA-best 57-16 record, earliest playoff clinch, and Shai Gilgeous-Alexander's MVP frontrunning amid Jalen Williams' injury return, despite Boston's 119-109 upset snapping OKC's 12-game win streak on March 25. San Antonio Spurs' 16% reflects Victor Wembanyama's dominant sophomore stats—leading blocks and rebounding—propelling their Southwest Division title and West No. 1 seed chase with nine games left. Boston Celtics at 11.8% leverage Eastern Conference contention (49-24) and Jaylen Brown's 31-point rally versus OKC, while Denver Nuggets' 8.5% hinges on Nikola Jokic's league-leading rebounds and assists in a bunched Western playoff race.", "context_requires_regen": true}, "liquidityClob": 8098580.77391, "enableOrderBook": true, "negRiskMarketID": "0x11e9a09023ace3097de216497c6fc01a57a57d63df7370543f288b40251dda00", "showAllOutcomes": true, "negRiskAugmented": false, "resolutionSource": "", "showMarketImages": false, "cumulativeMarkets": false, "pendingDeployment": false, "deployingTimestamp": "2025-06-23T15:28:44.417702Z", "automaticallyActive": true, "requiresTranslation": false}], "funded": false, "spread": 0.001, "volume": "25350912.14729484", "bestAsk": 0.001, "endDate": "2026-07-01T00:00:00Z", "feeType": null, "negRisk": true, "umaBond": "500", "approved": true, "archived": false, "featured": false, "outcomes": "[\"Yes\", \"No\"]", "question": "Will the Chicago Bulls win the 2026 NBA Finals?", "createdAt": "2025-06-19T18:23:38.667491Z", "deploying": false, "startDate": "2025-06-23T16:02:42.983826Z", "umaReward": "5", "updatedAt": "2026-03-29T06:43:33.067463Z", "volume1mo": 5070154.290501975, "volume1wk": 1352271.9670000018, "volume1yr": 25350912.147294898, "volumeNum": 25350912.14729484, "closedTime": "2026-03-28 07:41:55+00", "endDateIso": "2026-07-01", "questionID": "0x11e9a09023ace3097de216497c6fc01a57a57d63df7370543f288b40251dda16", "resolvedBy": "0x2F5e3684cb1F318ec51b00Edba38d79Ac2c0aA9d", "restricted": true, "rfqEnabled": false, "umaEndDate": "2026-03-28T07:41:55Z", "volume24hr": 180.29, "volumeClob": 25350912.14729484, "conditionId": "0xf374fb58698bccedf29399f9f5548a70370a11c0fece34f2570fb9b3885e8e5a", "description": "This market will resolve to “Yes” if the Chicago Bulls win the 2026 NBA Finals. Otherwise, this market will resolve to “No”.\n\nThis market will resolve to “No” if it becomes impossible for this team to win the 2026 NBA Finals based off the rules of the NBA.\n\nThe resolution source for this market will be information from the NBA.", "feesEnabled": false, "seriesColor": "", "clobTokenIds": "[\"101657448900324364213467059356648689270832606863187352286785694887095023173679\", \"95109892472860043698165831230345254090456546311265426162114533642591273071363\"]", "negRiskOther": false, "orderMinSize": 5, "startDateIso": "2025-06-23", "submitted_by": "0x91430CaD2d3975766499717fA0D66A78D814E5c5", "outcomePrices": "[\"0\", \"1\"]", "showGmpSeries": false, "volume1moClob": 5070154.290501975, "volume1wkClob": 1352271.9670000018, "volume1yrClob": 25350912.147294898, "groupItemTitle": "Chicago Bulls", "lastTradePrice": 0.001, "rewardsMinSize": 20, "showGmpOutcome": false, "volume24hrClob": 180.29, "acceptingOrders": false, "enableOrderBook": true, "negRiskMarketID": "0x11e9a09023ace3097de216497c6fc01a57a57d63df7370543f288b40251dda00", "clearBookOnStart": true, "hasReviewedDates": true, "manualActivation": false, "negRiskRequestID": "0x44221a0b742694c3114c7c93af03ea33e6ac61fa9e4854a019301ff03ff2f447", "resolutionSource": "", "rewardsMaxSpread": 3.5, "pendingDeployment": false, "deployingTimestamp": "2025-06-23T15:35:36.478958Z", "groupItemThreshold": "22", "marketMakerAddress": "", "automaticallyActive": true, "oneMonthPriceChange": -0.002, "requiresTranslation": false, "umaResolutionStatus": "resolved", "automaticallyResolved": true, "holdingRewardsEnabled": false, "orderPriceMinTickSize": 0.001, "umaResolutionStatuses": "[\"proposed\", \"resolved\"]", "acceptingOrdersTimestamp": "2025-06-23T16:02:15Z", "pagerDutyNotificationEnabled": false}</t>
         </is>
       </c>
       <c r="AJ2" s="1" t="n">
-        <v>46110.0765398214</v>
+        <v>46110.28125473107</v>
       </c>
       <c r="AK2" s="1" t="n">
-        <v>46110.07659220583</v>
+        <v>46110.28125473107</v>
       </c>
     </row>
     <row r="3">
@@ -784,7 +784,7 @@
         <v>45827.76644617892</v>
       </c>
       <c r="L3" s="1" t="n">
-        <v>46110.0758230725</v>
+        <v>46110.27999443856</v>
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" s="2" t="n">
@@ -812,34 +812,34 @@
         <v>1</v>
       </c>
       <c r="V3" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="W3" t="n">
         <v>0.011</v>
       </c>
-      <c r="W3" t="n">
-        <v>0.01</v>
-      </c>
       <c r="X3" t="n">
-        <v>0.012</v>
+        <v>0.013</v>
       </c>
       <c r="Y3" t="n">
         <v>0.002</v>
       </c>
       <c r="Z3" t="n">
-        <v>30216072.57437239</v>
+        <v>30312324.9928874</v>
       </c>
       <c r="AA3" t="n">
-        <v>30216072.57437239</v>
+        <v>30312324.9928874</v>
       </c>
       <c r="AB3" t="n">
-        <v>2316427.12051</v>
+        <v>2394730.649478</v>
       </c>
       <c r="AC3" t="n">
-        <v>11371823.45891905</v>
+        <v>11399629.82506505</v>
       </c>
       <c r="AD3" t="n">
-        <v>30216072.57437219</v>
+        <v>30312324.99288719</v>
       </c>
       <c r="AE3" t="n">
-        <v>314587.01121</v>
+        <v>316130.34592</v>
       </c>
       <c r="AF3" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>["0.011", "0.989"]</t>
+          <t>["0.012", "0.988"]</t>
         </is>
       </c>
       <c r="AH3" t="inlineStr">
@@ -858,14 +858,14 @@
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>{"id": "553882", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/nba-finals-points-leader-7g2ZEZvMXxLb.jpg", "slug": "will-the-charlotte-hornets-win-the-2026-nba-finals", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/nba-finals-points-leader-7g2ZEZvMXxLb.jpg", "ready": false, "active": true, "closed": false, "events": [{"id": "27830", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/nba-finals-points-leader-7g2ZEZvMXxLb.jpg", "slug": "2026-nba-champion", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/nba-finals-points-leader-7g2ZEZvMXxLb.jpg", "title": "2026 NBA Champion", "active": true, "closed": false, "sortBy": "price", "ticker": "2026-nba-champion", "volume": 207394956.867415, "endDate": "2026-07-01T00:00:00Z", "negRisk": true, "archived": false, "featured": false, "createdAt": "2025-06-19T18:23:26.785626Z", "deploying": false, "liquidity": 10039428.92563, "startDate": "2025-06-23T16:04:37.82012Z", "updatedAt": "2026-03-29T01:49:32.895725Z", "volume1mo": 73091497.38166507, "volume1wk": 17785304.81427103, "volume1yr": 207394956.86741585, "restricted": true, "volume24hr": 2335162.860974, "competitive": 0.9846153846153846, "description": "This market is to predict the winner of the 2025–26 NBA Finals.", "commentCount": 259, "creationDate": "2025-06-23T16:04:37.820118Z", "gmpChartMode": "default", "openInterest": 2706230.92922, "enableNegRisk": true, "eventMetadata": {"context_updated_at": "2026-03-29T01:46:27.538Z", "context_description": "Oklahoma City Thunder lead Polymarket's 2026 NBA Champion market at 37.5% implied probability, reflecting their league-best 57-16 record and first-to-clinch playoff berth in the stacked Western Conference, bolstered by Shai Gilgeous-Alexander's MVP-caliber play and a dominant 131-113 win over Chicago on March 27 featuring a 22-0 second-half run. San Antonio Spurs trail at 15.6% amid a scorching seven-game win streak—including a 123-98 rout of Memphis on March 25—fueled by Victor Wembanyama's MVP candidacy and the NBA's deepest roster, closing the gap on OKC in standings (55-18). Boston Celtics hold third at 11.5% with a solid 49-24 East mark, though Detroit Pistons' surge (53-20) intensifies conference finals path; Denver Nuggets (8.5%) rely on Nikola Jokić's historic triple-doubles despite middling 46-28 standing. Trader consensus prices emphasize West dominance, health, and late-season momentum with under 10 games left.", "context_requires_regen": true}, "liquidityClob": 10039428.92563, "enableOrderBook": true, "negRiskMarketID": "0x11e9a09023ace3097de216497c6fc01a57a57d63df7370543f288b40251dda00", "showAllOutcomes": true, "negRiskAugmented": false, "resolutionSource": "", "showMarketImages": false, "cumulativeMarkets": false, "pendingDeployment": false, "deployingTimestamp": "2025-06-23T15:28:44.417702Z", "automaticallyActive": true, "requiresTranslation": false}], "funded": false, "spread": 0.002, "volume": "30216072.574372392", "bestAsk": 0.012, "bestBid": 0.01, "endDate": "2026-07-01T00:00:00Z", "feeType": null, "negRisk": true, "umaBond": "500", "approved": true, "archived": false, "featured": false, "outcomes": "[\"Yes\", \"No\"]", "question": "Will the Charlotte Hornets win the 2026 NBA Finals?", "createdAt": "2025-06-19T18:23:40.949859Z", "deploying": false, "liquidity": "314587.01121", "startDate": "2025-06-23T16:02:47.87066Z", "umaReward": "5", "updatedAt": "2026-03-29T01:49:11.113464Z", "volume1mo": 11371823.458919052, "volume1wk": 2316427.1205100003, "volume1yr": 30216072.574372187, "volumeNum": 30216072.574372392, "endDateIso": "2026-07-01", "questionID": "0x11e9a09023ace3097de216497c6fc01a57a57d63df7370543f288b40251dda1a", "resolvedBy": "0x2F5e3684cb1F318ec51b00Edba38d79Ac2c0aA9d", "restricted": true, "rfqEnabled": false, "volume24hr": 499620.997428, "volumeClob": 30216072.574372392, "competitive": 0.8070236885663306, "conditionId": "0xc58cfb7397c4f3f803f5c20135cafa7f6d2c87cf3bb1e6138042b95d828e1866", "description": "This market will resolve to “Yes” if the Charlotte Hornets win the 2026 NBA Finals. Otherwise, this market will resolve to “No”.\n\nThis market will resolve to “No” if it becomes impossible for this team to win the 2026 NBA Finals based off the rules of the NBA.\n\nThe resolution source for this market will be information from the NBA.", "feesEnabled": false, "seriesColor": "", "clobTokenIds": "[\"56958503032603479474712760211473691965846495282533669255954105717594026846100\", \"65993209531308632524221798569537933773833000068656072810215460807745426846637\"]", "liquidityNum": 314587.01121, "negRiskOther": false, "orderMinSize": 5, "startDateIso": "2025-06-23", "submitted_by": "0x91430CaD2d3975766499717fA0D66A78D814E5c5", "liquidityClob": 314587.01121, "outcomePrices": "[\"0.011\", \"0.989\"]", "showGmpSeries": false, "volume1moClob": 11371823.458919052, "volume1wkClob": 2316427.1205100003, "volume1yrClob": 30216072.574372187, "groupItemTitle": "Charlotte Hornets", "lastTradePrice": 0.011, "rewardsMinSize": 20, "showGmpOutcome": false, "volume24hrClob": 499620.997428, "acceptingOrders": true, "enableOrderBook": true, "negRiskMarketID": "0x11e9a09023ace3097de216497c6fc01a57a57d63df7370543f288b40251dda00", "clearBookOnStart": true, "hasReviewedDates": true, "manualActivation": false, "negRiskRequestID": "0xefa48886269a0abc9cbf3e343ad122e28c62f9aa1c922b6f5804a685fcc1d681", "resolutionSource": "", "rewardsMaxSpread": 3.5, "oneDayPriceChange": 0.0005, "pendingDeployment": false, "deployingTimestamp": "2025-06-23T15:35:36.484193Z", "groupItemThreshold": "26", "marketMakerAddress": "", "oneHourPriceChange": 0.0005, "oneWeekPriceChange": -0.0035, "automaticallyActive": true, "oneMonthPriceChange": 0.0055, "requiresTranslation": false, "holdingRewardsEnabled": false, "orderPriceMinTickSize": 0.001, "umaResolutionStatuses": "[]", "acceptingOrdersTimestamp": "2025-06-23T16:02:19Z", "pagerDutyNotificationEnabled": false}</t>
+          <t>{"id": "553882", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/nba-finals-points-leader-7g2ZEZvMXxLb.jpg", "slug": "will-the-charlotte-hornets-win-the-2026-nba-finals", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/nba-finals-points-leader-7g2ZEZvMXxLb.jpg", "ready": false, "active": true, "closed": false, "events": [{"id": "27830", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/nba-finals-points-leader-7g2ZEZvMXxLb.jpg", "slug": "2026-nba-champion", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/nba-finals-points-leader-7g2ZEZvMXxLb.jpg", "title": "2026 NBA Champion", "active": true, "closed": false, "sortBy": "price", "ticker": "2026-nba-champion", "volume": 207959072.18360305, "endDate": "2026-07-01T00:00:00Z", "negRisk": true, "archived": false, "featured": false, "createdAt": "2025-06-19T18:23:26.785626Z", "deploying": false, "liquidity": 8098580.77391, "startDate": "2025-06-23T16:04:37.82012Z", "updatedAt": "2026-03-29T06:43:33.736055Z", "volume1mo": 72985303.69146004, "volume1wk": 17899490.499662023, "volume1yr": 207959072.18360385, "restricted": true, "volume24hr": 2322731.1560189994, "competitive": 0.9846153846153846, "description": "This market is to predict the winner of the 2025–26 NBA Finals.", "commentCount": 260, "creationDate": "2025-06-23T16:04:37.820118Z", "gmpChartMode": "default", "openInterest": 2787127.0686719995, "enableNegRisk": true, "eventMetadata": {"context_updated_at": "2026-03-29T06:30:50.883Z", "context_description": "Oklahoma City Thunder command 37.5% implied probability as 2026 NBA champions per trader consensus, fueled by their NBA-best 57-16 record, earliest playoff clinch, and Shai Gilgeous-Alexander's MVP frontrunning amid Jalen Williams' injury return, despite Boston's 119-109 upset snapping OKC's 12-game win streak on March 25. San Antonio Spurs' 16% reflects Victor Wembanyama's dominant sophomore stats—leading blocks and rebounding—propelling their Southwest Division title and West No. 1 seed chase with nine games left. Boston Celtics at 11.8% leverage Eastern Conference contention (49-24) and Jaylen Brown's 31-point rally versus OKC, while Denver Nuggets' 8.5% hinges on Nikola Jokic's league-leading rebounds and assists in a bunched Western playoff race.", "context_requires_regen": true}, "liquidityClob": 8098580.77391, "enableOrderBook": true, "negRiskMarketID": "0x11e9a09023ace3097de216497c6fc01a57a57d63df7370543f288b40251dda00", "showAllOutcomes": true, "negRiskAugmented": false, "resolutionSource": "", "showMarketImages": false, "cumulativeMarkets": false, "pendingDeployment": false, "deployingTimestamp": "2025-06-23T15:28:44.417702Z", "automaticallyActive": true, "requiresTranslation": false}], "funded": false, "spread": 0.002, "volume": "30312324.9928874", "bestAsk": 0.013, "bestBid": 0.011, "endDate": "2026-07-01T00:00:00Z", "feeType": null, "negRisk": true, "umaBond": "500", "approved": true, "archived": false, "featured": false, "outcomes": "[\"Yes\", \"No\"]", "question": "Will the Charlotte Hornets win the 2026 NBA Finals?", "createdAt": "2025-06-19T18:23:40.949859Z", "deploying": false, "liquidity": "316130.34592", "startDate": "2025-06-23T16:02:47.87066Z", "umaReward": "5", "updatedAt": "2026-03-29T06:43:11.519491Z", "volume1mo": 11399629.825065047, "volume1wk": 2394730.649478, "volume1yr": 30312324.99288719, "volumeNum": 30312324.9928874, "endDateIso": "2026-07-01", "questionID": "0x11e9a09023ace3097de216497c6fc01a57a57d63df7370543f288b40251dda1a", "resolvedBy": "0x2F5e3684cb1F318ec51b00Edba38d79Ac2c0aA9d", "restricted": true, "rfqEnabled": false, "volume24hr": 494910.5429529999, "volumeClob": 30312324.9928874, "competitive": 0.807660498294221, "conditionId": "0xc58cfb7397c4f3f803f5c20135cafa7f6d2c87cf3bb1e6138042b95d828e1866", "description": "This market will resolve to “Yes” if the Charlotte Hornets win the 2026 NBA Finals. Otherwise, this market will resolve to “No”.\n\nThis market will resolve to “No” if it becomes impossible for this team to win the 2026 NBA Finals based off the rules of the NBA.\n\nThe resolution source for this market will be information from the NBA.", "feesEnabled": false, "seriesColor": "", "clobTokenIds": "[\"56958503032603479474712760211473691965846495282533669255954105717594026846100\", \"65993209531308632524221798569537933773833000068656072810215460807745426846637\"]", "liquidityNum": 316130.34592, "negRiskOther": false, "orderMinSize": 5, "startDateIso": "2025-06-23", "submitted_by": "0x91430CaD2d3975766499717fA0D66A78D814E5c5", "liquidityClob": 316130.34592, "outcomePrices": "[\"0.012\", \"0.988\"]", "showGmpSeries": false, "volume1moClob": 11399629.825065047, "volume1wkClob": 2394730.649478, "volume1yrClob": 30312324.99288719, "groupItemTitle": "Charlotte Hornets", "lastTradePrice": 0.012, "rewardsMinSize": 20, "showGmpOutcome": false, "volume24hrClob": 494910.5429529999, "acceptingOrders": true, "enableOrderBook": true, "negRiskMarketID": "0x11e9a09023ace3097de216497c6fc01a57a57d63df7370543f288b40251dda00", "clearBookOnStart": true, "hasReviewedDates": true, "manualActivation": false, "negRiskRequestID": "0xefa48886269a0abc9cbf3e343ad122e28c62f9aa1c922b6f5804a685fcc1d681", "resolutionSource": "", "rewardsMaxSpread": 3.5, "oneDayPriceChange": 0.0005, "pendingDeployment": false, "deployingTimestamp": "2025-06-23T15:35:36.484193Z", "groupItemThreshold": "26", "marketMakerAddress": "", "oneHourPriceChange": 0.0005, "oneWeekPriceChange": -0.0035, "automaticallyActive": true, "oneMonthPriceChange": 0.0055, "requiresTranslation": false, "holdingRewardsEnabled": false, "orderPriceMinTickSize": 0.001, "umaResolutionStatuses": "[]", "acceptingOrdersTimestamp": "2025-06-23T16:02:19Z", "pagerDutyNotificationEnabled": false}</t>
         </is>
       </c>
       <c r="AJ3" s="1" t="n">
-        <v>46110.0765398214</v>
+        <v>46110.28125473107</v>
       </c>
       <c r="AK3" s="1" t="n">
-        <v>46110.07659220583</v>
+        <v>46110.28125473107</v>
       </c>
     </row>
     <row r="4">
@@ -914,7 +914,7 @@
         <v>45840.70481185071</v>
       </c>
       <c r="L4" s="1" t="n">
-        <v>46110.07590366778</v>
+        <v>46110.27998155871</v>
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" s="2" t="n">
@@ -945,31 +945,31 @@
         <v>0.002</v>
       </c>
       <c r="W4" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="X4" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="Y4" t="n">
         <v>0.001</v>
       </c>
       <c r="Z4" t="n">
-        <v>25981212.59053205</v>
+        <v>26045284.43803205</v>
       </c>
       <c r="AA4" t="n">
-        <v>25981212.59053205</v>
+        <v>26045284.43803205</v>
       </c>
       <c r="AB4" t="n">
-        <v>1595498.739999992</v>
+        <v>1617233.064499992</v>
       </c>
       <c r="AC4" t="n">
-        <v>4911447.520000112</v>
+        <v>4956686.286000114</v>
       </c>
       <c r="AD4" t="n">
-        <v>25981212.59055207</v>
+        <v>26045284.43805207</v>
       </c>
       <c r="AE4" t="n">
-        <v>1415610.51872</v>
+        <v>1401452.95025</v>
       </c>
       <c r="AF4" t="inlineStr">
         <is>
@@ -978,7 +978,7 @@
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>["0.0015", "0.9985"]</t>
+          <t>["0.0025", "0.9975"]</t>
         </is>
       </c>
       <c r="AH4" t="inlineStr">
@@ -988,14 +988,14 @@
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>{"id": "558960", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/will-uzbekistan-win-the-2026-fifa-world-cup-773-YUDww6rLHD3U.jpg", "slug": "will-uzbekistan-win-the-2026-fifa-world-cup-773", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/will-uzbekistan-win-the-2026-fifa-world-cup-773-YUDww6rLHD3U.jpg", "ready": false, "active": true, "closed": false, "events": [{"id": "30615", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/2026-fifa-world-cup-winner-595-8rgoVIZnbKgL.png", "slug": "2026-fifa-world-cup-winner-595", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/2026-fifa-world-cup-winner-595-8rgoVIZnbKgL.png", "title": "2026 FIFA World Cup Winner ", "active": true, "closed": false, "sortBy": "price", "ticker": "2026-fifa-world-cup-winner-595", "volume": 405091232.4410685, "endDate": "2026-07-20T00:00:00Z", "negRisk": true, "archived": false, "featured": true, "createdAt": "2025-07-02T16:54:39.838289Z", "deploying": false, "liquidity": 47505630.74751, "startDate": "2025-07-02T22:28:24.564603Z", "updatedAt": "2026-03-29T01:49:40.202921Z", "volume1mo": 193397140.5715902, "volume1wk": 59481504.43325691, "volume1yr": 405091232.4410212, "restricted": true, "volume24hr": 12099234.407564001, "competitive": 0.8950097612002081, "description": "This market will resolve according to the national team that wins the 2026 FIFA World Cup.\n\nIf at any point it becomes impossible for this team to win the FIFA World Cup based on the rules of FIFA (e.g., they are eliminated in the knockout stage), this market will resolve immediately to “No”.\n\nIf the 2026 FIFA World Cup is permanently canceled or has not been completed by October 13, 2026, 11:59 PM this market will resolve to “Other”.\n\nThe primary resolution source will be official information from FIFA, however, a consensus of credible reporting may also be used.", "commentCount": 446, "creationDate": "2025-07-02T22:28:24.564583Z", "gmpChartMode": "default", "openInterest": 5192277.364946, "enableNegRisk": true, "estimateValue": false, "eventMetadata": {"context_updated_at": "2026-03-29T01:46:27.457Z", "context_description": "Spain holds a slim edge in trader consensus at 15.8% implied probability to win the 2026 FIFA World Cup, buoyed by their dominant Euro 2024 triumph and flawless UEFA qualifying campaign, capped by a 3-0 friendly rout of Serbia on March 28 that showcased Lamine Yamal and Pedri's attacking flair. England (12.8%), France (10.8%), Argentina (9.9%), and Brazil (8.6%) trail closely, their probabilities bunched amid CONMEBOL powerhouses securing direct spots and the December 2025 group draw shielding elite seeds from early clashes until knockout rounds. Recent UEFA playoffs (Italy's 2-0 win over Northern Ireland, Bosnia's penalty advance past Wales on March 26) affirm Europe's depth, while no major injuries or upsets have emerged to separate the pack, keeping the race competitively tight with host-nation factors and expanded 48-team format adding unpredictability.", "context_requires_regen": true}, "featuredOrder": 11, "liquidityClob": 47505630.74751, "enableOrderBook": true, "negRiskMarketID": "0xb5c32a9acd39848acad4913ac4cd49c5de2afcc9d23a8a7ba2419375fab87400", "showAllOutcomes": true, "negRiskAugmented": true, "resolutionSource": "", "showMarketImages": true, "cumulativeMarkets": false, "pendingDeployment": false, "deployingTimestamp": "2025-07-02T22:06:00.953755Z", "automaticallyActive": true, "requiresTranslation": false}], "funded": false, "spread": 0.001, "volume": "25981212.590532053", "bestAsk": 0.002, "bestBid": 0.001, "endDate": "2026-07-20T00:00:00Z", "feeType": null, "negRisk": true, "umaBond": "500", "approved": true, "archived": false, "featured": false, "outcomes": "[\"Yes\", \"No\"]", "question": "Will Uzbekistan win the 2026 FIFA World Cup?", "createdAt": "2025-07-02T16:54:55.743901Z", "deploying": false, "liquidity": "1415610.51872", "startDate": "2025-07-02T22:27:23.588Z", "umaReward": "5", "updatedAt": "2026-03-29T01:49:18.076896Z", "volume1mo": 4911447.520000112, "volume1wk": 1595498.7399999916, "volume1yr": 25981212.590552066, "volumeNum": 25981212.590532053, "endDateIso": "2026-07-20", "questionID": "0xb5c32a9acd39848acad4913ac4cd49c5de2afcc9d23a8a7ba2419375fab87419", "resolvedBy": "0x2F5e3684cb1F318ec51b00Edba38d79Ac2c0aA9d", "restricted": true, "rfqEnabled": false, "volume24hr": 375747.834, "volumeClob": 25981212.590532053, "competitive": 0.8009597099244316, "conditionId": "0x965ebc5d79eb1ec02cad67245a44b9e45b33359018f013fb6cf81d5bbf7bcc8d", "description": "This market will resolve according to the national team that wins the 2026 FIFA World Cup.\n\nIf at any point it becomes impossible for this team to win the FIFA World Cup based on the rules of FIFA (e.g., they are eliminated in the knockout stage), this market will resolve immediately to “No”.\n\nIf the 2026 FIFA World Cup is permanently canceled or has not been completed by October 13, 2026, 11:59 PM this market will resolve to “Other”.\n\nThe primary resolution source will be official information from FIFA, however, a consensus of credible reporting may also be used.", "feesEnabled": false, "seriesColor": "", "clobTokenIds": "[\"90538013438399246674125939147272424357773921253199632436930218305581040235987\", \"105754735859803813986361714630753276237891536292440584153365249756008425623608\"]", "liquidityNum": 1415610.51872, "negRiskOther": false, "orderMinSize": 5, "startDateIso": "2025-07-02", "submitted_by": "0x91430CaD2d3975766499717fA0D66A78D814E5c5", "liquidityClob": 1415610.51872, "outcomePrices": "[\"0.0015\", \"0.9985\"]", "showGmpSeries": false, "volume1moClob": 4911447.520000112, "volume1wkClob": 1595498.7399999916, "volume1yrClob": 25981212.590552066, "customLiveness": 0, "groupItemTitle": "Uzbekistan", "lastTradePrice": 0.002, "rewardsMinSize": 20, "showGmpOutcome": false, "volume24hrClob": 375747.834, "acceptingOrders": true, "enableOrderBook": true, "negRiskMarketID": "0xb5c32a9acd39848acad4913ac4cd49c5de2afcc9d23a8a7ba2419375fab87400", "clearBookOnStart": true, "hasReviewedDates": true, "manualActivation": true, "negRiskRequestID": "0x755362c84e0c147aff0edd7f1115b18f94d4191484d4b9d8c81668b544110d5f", "resolutionSource": "", "rewardsMaxSpread": 3.5, "pendingDeployment": false, "deployingTimestamp": "2025-07-02T22:06:41.865719Z", "groupItemThreshold": "24", "marketMakerAddress": "", "oneWeekPriceChange": -0.001, "automaticallyActive": true, "oneMonthPriceChange": -0.001, "requiresTranslation": false, "holdingRewardsEnabled": true, "orderPriceMinTickSize": 0.001, "umaResolutionStatuses": "[]", "acceptingOrdersTimestamp": "2025-07-02T22:26:55Z", "pagerDutyNotificationEnabled": false}</t>
+          <t>{"id": "558960", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/will-uzbekistan-win-the-2026-fifa-world-cup-773-YUDww6rLHD3U.jpg", "slug": "will-uzbekistan-win-the-2026-fifa-world-cup-773", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/will-uzbekistan-win-the-2026-fifa-world-cup-773-YUDww6rLHD3U.jpg", "ready": false, "active": true, "closed": false, "events": [{"id": "30615", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/2026-fifa-world-cup-winner-595-8rgoVIZnbKgL.png", "slug": "2026-fifa-world-cup-winner-595", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/2026-fifa-world-cup-winner-595-8rgoVIZnbKgL.png", "title": "2026 FIFA World Cup Winner ", "active": true, "closed": false, "sortBy": "price", "ticker": "2026-fifa-world-cup-winner-595", "volume": 407779862.6814054, "endDate": "2026-07-20T00:00:00Z", "negRisk": true, "archived": false, "featured": true, "createdAt": "2025-07-02T16:54:39.838289Z", "deploying": false, "liquidity": 47470508.90118, "startDate": "2025-07-02T22:28:24.564603Z", "updatedAt": "2026-03-29T06:44:14.561068Z", "volume1mo": 194563572.88009733, "volume1wk": 60710538.365675904, "volume1yr": 407779862.6813582, "restricted": true, "volume24hr": 11103417.103119997, "competitive": 0.8952840019911116, "description": "This market will resolve according to the national team that wins the 2026 FIFA World Cup.\n\nIf at any point it becomes impossible for this team to win the FIFA World Cup based on the rules of FIFA (e.g., they are eliminated in the knockout stage), this market will resolve immediately to “No”.\n\nIf the 2026 FIFA World Cup is permanently canceled or has not been completed by October 13, 2026, 11:59 PM this market will resolve to “Other”.\n\nThe primary resolution source will be official information from FIFA, however, a consensus of credible reporting may also be used.", "commentCount": 447, "creationDate": "2025-07-02T22:28:24.564583Z", "gmpChartMode": "default", "openInterest": 4998549.925569001, "enableNegRisk": true, "estimateValue": false, "eventMetadata": {"context_updated_at": "2026-03-29T06:31:01.791Z", "context_description": "Spain tops trader consensus at 15.8% implied probability for the 2026 FIFA World Cup, buoyed by their No. 1 FIFA ranking after a dominant UEFA qualifying campaign capped by a 2-0 clean-sheet win over Georgia on March 26. England follows closely at 12.8% following a 5-0 thrashing of Latvia in Group K qualifiers, while France (10.8%) leads Group D with recent away victories like 3-1 at Azerbaijan. Argentina (9.9%) clinched top spot in CONMEBOL standings unbeaten, ahead of Brazil (8.6%) despite their mid-table finish, highlighting South American depth. The bunched odds reflect parity among group leaders, peaking golden generations—Spain's Yamal-led youth, Mbappé's France, Messi's farewell push—and bracket rules separating elites until semifinals in the expanded 48-team format.", "context_requires_regen": true}, "featuredOrder": 11, "liquidityClob": 47470508.90118, "enableOrderBook": true, "negRiskMarketID": "0xb5c32a9acd39848acad4913ac4cd49c5de2afcc9d23a8a7ba2419375fab87400", "showAllOutcomes": true, "negRiskAugmented": true, "resolutionSource": "", "showMarketImages": true, "cumulativeMarkets": false, "pendingDeployment": false, "deployingTimestamp": "2025-07-02T22:06:00.953755Z", "automaticallyActive": true, "requiresTranslation": false}], "funded": false, "spread": 0.001, "volume": "26045284.43803205", "bestAsk": 0.003, "bestBid": 0.002, "endDate": "2026-07-20T00:00:00Z", "feeType": null, "negRisk": true, "umaBond": "500", "approved": true, "archived": false, "featured": false, "outcomes": "[\"Yes\", \"No\"]", "question": "Will Uzbekistan win the 2026 FIFA World Cup?", "createdAt": "2025-07-02T16:54:55.743901Z", "deploying": false, "liquidity": "1401452.95025", "startDate": "2025-07-02T22:27:23.588Z", "umaReward": "5", "updatedAt": "2026-03-29T06:43:10.406673Z", "volume1mo": 4956686.286000114, "volume1wk": 1617233.0644999917, "volume1yr": 26045284.438052066, "volumeNum": 26045284.43803205, "endDateIso": "2026-07-20", "questionID": "0xb5c32a9acd39848acad4913ac4cd49c5de2afcc9d23a8a7ba2419375fab87419", "resolvedBy": "0x2F5e3684cb1F318ec51b00Edba38d79Ac2c0aA9d", "restricted": true, "rfqEnabled": false, "volume24hr": 402483.28250000003, "volumeClob": 26045284.43803205, "competitive": 0.8015991903848178, "conditionId": "0x965ebc5d79eb1ec02cad67245a44b9e45b33359018f013fb6cf81d5bbf7bcc8d", "description": "This market will resolve according to the national team that wins the 2026 FIFA World Cup.\n\nIf at any point it becomes impossible for this team to win the FIFA World Cup based on the rules of FIFA (e.g., they are eliminated in the knockout stage), this market will resolve immediately to “No”.\n\nIf the 2026 FIFA World Cup is permanently canceled or has not been completed by October 13, 2026, 11:59 PM this market will resolve to “Other”.\n\nThe primary resolution source will be official information from FIFA, however, a consensus of credible reporting may also be used.", "feesEnabled": false, "seriesColor": "", "clobTokenIds": "[\"90538013438399246674125939147272424357773921253199632436930218305581040235987\", \"105754735859803813986361714630753276237891536292440584153365249756008425623608\"]", "liquidityNum": 1401452.95025, "negRiskOther": false, "orderMinSize": 5, "startDateIso": "2025-07-02", "submitted_by": "0x91430CaD2d3975766499717fA0D66A78D814E5c5", "liquidityClob": 1401452.95025, "outcomePrices": "[\"0.0025\", \"0.9975\"]", "showGmpSeries": false, "volume1moClob": 4956686.286000114, "volume1wkClob": 1617233.0644999917, "volume1yrClob": 26045284.438052066, "customLiveness": 0, "groupItemTitle": "Uzbekistan", "lastTradePrice": 0.002, "rewardsMinSize": 20, "showGmpOutcome": false, "volume24hrClob": 402483.28250000003, "acceptingOrders": true, "enableOrderBook": true, "negRiskMarketID": "0xb5c32a9acd39848acad4913ac4cd49c5de2afcc9d23a8a7ba2419375fab87400", "clearBookOnStart": true, "hasReviewedDates": true, "manualActivation": true, "negRiskRequestID": "0x755362c84e0c147aff0edd7f1115b18f94d4191484d4b9d8c81668b544110d5f", "resolutionSource": "", "rewardsMaxSpread": 3.5, "pendingDeployment": false, "deployingTimestamp": "2025-07-02T22:06:41.865719Z", "groupItemThreshold": "24", "marketMakerAddress": "", "oneWeekPriceChange": -0.001, "automaticallyActive": true, "oneMonthPriceChange": -0.001, "requiresTranslation": false, "holdingRewardsEnabled": true, "orderPriceMinTickSize": 0.001, "umaResolutionStatuses": "[]", "acceptingOrdersTimestamp": "2025-07-02T22:26:55Z", "pagerDutyNotificationEnabled": false}</t>
         </is>
       </c>
       <c r="AJ4" s="1" t="n">
-        <v>46110.0765398214</v>
+        <v>46110.28125473107</v>
       </c>
       <c r="AK4" s="1" t="n">
-        <v>46110.07659220583</v>
+        <v>46110.28125473107</v>
       </c>
     </row>
     <row r="5">
@@ -1043,7 +1043,7 @@
         <v>45841.85912181914</v>
       </c>
       <c r="L5" s="1" t="n">
-        <v>46110.07586185105</v>
+        <v>46110.28003235196</v>
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" s="2" t="n">
@@ -1083,22 +1083,22 @@
         <v>0.001</v>
       </c>
       <c r="Z5" t="n">
-        <v>24183448.13280705</v>
+        <v>24231964.76713505</v>
       </c>
       <c r="AA5" t="n">
-        <v>24183448.13280705</v>
+        <v>24231964.76713505</v>
       </c>
       <c r="AB5" t="n">
-        <v>1580267.287608907</v>
+        <v>1574246.477223908</v>
       </c>
       <c r="AC5" t="n">
-        <v>6262651.365774389</v>
+        <v>6280163.686772391</v>
       </c>
       <c r="AD5" t="n">
-        <v>24183448.13280332</v>
+        <v>24231964.76713132</v>
       </c>
       <c r="AE5" t="n">
-        <v>1613570.36251</v>
+        <v>1596308.44339</v>
       </c>
       <c r="AF5" t="inlineStr">
         <is>
@@ -1117,14 +1117,14 @@
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>{"id": "559664", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/Raphael_Warnock.png", "slug": "will-raphael-warnock-win-the-2028-democratic-presidential-nomination-914", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/Raphael_Warnock.png", "ready": false, "active": true, "closed": false, "events": [{"id": "30829", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/democrats+2028+donkey.png", "slug": "democratic-presidential-nominee-2028", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/democrats+2028+donkey.png", "title": "Democratic Presidential Nominee 2028", "active": true, "closed": false, "sortBy": "price", "ticker": "democratic-presidential-nominee-2028", "volume": 929408692.9919622, "endDate": "2028-11-07T00:00:00Z", "negRisk": true, "archived": false, "featured": true, "createdAt": "2025-07-03T20:36:57.824243Z", "deploying": false, "liquidity": 44060833.8747, "startDate": "2025-07-11T18:41:17.827458Z", "startTime": "2028-11-07T12:00:00Z", "updatedAt": "2026-03-29T01:49:40.20413Z", "volume1mo": 201497523.6404877, "volume1wk": 53094243.130744666, "volume1yr": 929408692.9919566, "restricted": true, "volume24hr": 4958628.24913, "competitive": 0.9382691608050256, "countryName": "U.S.", "description": "This market will resolve to “Yes” if the named individual wins and accepts the 2028 nomination of the Democratic Party for U.S. president. Otherwise, this market will resolve to “No”.\n\nThe resolution source for this market will be a consensus of official Democratic Party sources.\n\nAny replacement of the democratic nominee before election day will not change the resolution of the market.", "commentCount": 616, "creationDate": "2025-07-11T18:41:17.827389Z", "electionType": "Democratic Nomination", "gmpChartMode": "default", "openInterest": 10925893.814415, "enableNegRisk": true, "estimateValue": false, "eventMetadata": {"context_updated_at": "2026-03-29T01:46:24.319Z", "context_description": "California Governor Gavin Newsom leads Polymarket's Democratic presidential nominee 2028 odds at 24.3% implied probability, driven by his March book tour in New Hampshire—testing early primary waters—and a March 12 California poll showing a 14-point edge over Kamala Harris, bolstering his executive experience and national anti-Trump profile amid party reckoning post-2024. Rep. Alexandria Ocasio-Cortez holds 8.3% on progressive grassroots energy and social media reach, though centrist groups like Third Way mobilized in March against left-wing frontrunners to prioritize electability. Sen. Jon Ossoff's 5.8% stems from Georgia battleground wins appealing to swing-state math. This fragmented field, with no outcome above 25%, could consolidate via 2026 midterm performances, fundraising dominance, key endorsements, or polling shifts favoring incumbents or moderates.", "context_requires_regen": true}, "featuredOrder": 15, "liquidityClob": 44060833.8747, "enableOrderBook": true, "negRiskMarketID": "0x2c3d7e0eee6f058be3006baabf0d54a07da254ba47fe6e3e095e7990c7814700", "showAllOutcomes": true, "negRiskAugmented": true, "resolutionSource": "", "showMarketImages": true, "cumulativeMarkets": false, "pendingDeployment": false, "deployingTimestamp": "2025-07-11T18:14:44.108448Z", "automaticallyActive": true, "requiresTranslation": false}], "funded": false, "spread": 0.001, "volume": "24183448.132807046", "bestAsk": 0.006, "bestBid": 0.005, "endDate": "2028-11-07T00:00:00Z", "feeType": null, "negRisk": true, "umaBond": "25000", "approved": true, "archived": false, "featured": false, "outcomes": "[\"Yes\", \"No\"]", "question": "Will Raphael Warnock win the 2028 Democratic presidential nomination?", "createdAt": "2025-07-03T20:37:08.125174Z", "deploying": false, "liquidity": "1613570.36251", "startDate": "2025-07-11T18:36:11.106Z", "umaReward": "10", "updatedAt": "2026-03-29T01:49:14.463931Z", "volume1mo": 6262651.365774389, "volume1wk": 1580267.2876089069, "volume1yr": 24183448.13280332, "volumeNum": 24183448.132807046, "endDateIso": "2028-11-07", "questionID": "0x2c3d7e0eee6f058be3006baabf0d54a07da254ba47fe6e3e095e7990c781470c", "resolvedBy": "0x2F5e3684cb1F318ec51b00Edba38d79Ac2c0aA9d", "restricted": true, "rfqEnabled": false, "volume24hr": 262245.774253, "volumeClob": 24183448.132807046, "competitive": 0.8035160254240507, "conditionId": "0xdce84960dce38aa4a5800a5eba7c9ac34d2ce49ba9d44c42572c472d468af264", "description": "This market will resolve to “Yes” if the named individual wins and accepts the 2028 nomination of the Democratic Party for U.S. president. Otherwise, this market will resolve to “No”.\n\nThe resolution source for this market will be a consensus of official Democratic Party sources.\n\nAny replacement of the democratic nominee before election day will not change the resolution of the market.", "feesEnabled": false, "seriesColor": "", "clobTokenIds": "[\"52310257194926233099477326083312959938983447523839326865869372741334281264830\", \"88403451835230950222119400360490338078378790763472355557584611572247419676051\"]", "liquidityNum": 1613570.36251, "negRiskOther": false, "orderMinSize": 5, "startDateIso": "2025-07-11", "submitted_by": "0x91430CaD2d3975766499717fA0D66A78D814E5c5", "liquidityClob": 1613570.36251, "outcomePrices": "[\"0.0055\", \"0.9945\"]", "showGmpSeries": false, "volume1moClob": 6262651.365774389, "volume1wkClob": 1580267.2876089069, "volume1yrClob": 24183448.13280332, "customLiveness": 0, "groupItemTitle": "Raphael Warnock", "lastTradePrice": 0.005, "rewardsMinSize": 20, "showGmpOutcome": false, "volume24hrClob": 262245.774253, "acceptingOrders": true, "enableOrderBook": true, "negRiskMarketID": "0x2c3d7e0eee6f058be3006baabf0d54a07da254ba47fe6e3e095e7990c7814700", "clearBookOnStart": true, "hasReviewedDates": true, "manualActivation": false, "negRiskRequestID": "0x7582e1feb071a286ac4803ff6555fe830cded5480ede75b13f5de7325842e4e8", "resolutionSource": "", "rewardsMaxSpread": 3.5, "pendingDeployment": false, "deployingTimestamp": "2025-07-11T18:15:13.626487Z", "groupItemThreshold": "12", "marketMakerAddress": "", "oneWeekPriceChange": 0.001, "automaticallyActive": true, "oneMonthPriceChange": 0.003, "requiresTranslation": false, "holdingRewardsEnabled": true, "orderPriceMinTickSize": 0.001, "umaResolutionStatuses": "[]", "acceptingOrdersTimestamp": "2025-07-11T18:35:48Z", "pagerDutyNotificationEnabled": false}</t>
+          <t>{"id": "559664", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/Raphael_Warnock.png", "slug": "will-raphael-warnock-win-the-2028-democratic-presidential-nomination-914", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/Raphael_Warnock.png", "ready": false, "active": true, "closed": false, "events": [{"id": "30829", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/democrats+2028+donkey.png", "slug": "democratic-presidential-nominee-2028", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/democrats+2028+donkey.png", "title": "Democratic Presidential Nominee 2028", "active": true, "closed": false, "sortBy": "price", "ticker": "democratic-presidential-nominee-2028", "volume": 930647837.2445823, "endDate": "2028-11-07T00:00:00Z", "negRisk": true, "archived": false, "featured": true, "createdAt": "2025-07-03T20:36:57.824243Z", "deploying": false, "liquidity": 43770146.56328, "startDate": "2025-07-11T18:41:17.827458Z", "startTime": "2028-11-07T12:00:00Z", "updatedAt": "2026-03-29T06:44:46.607657Z", "volume1mo": 201648772.32079622, "volume1wk": 51178107.61075467, "volume1yr": 930647837.2445767, "restricted": true, "volume24hr": 5365195.267472, "competitive": 0.9382691608050256, "countryName": "U.S.", "description": "This market will resolve to “Yes” if the named individual wins and accepts the 2028 nomination of the Democratic Party for U.S. president. Otherwise, this market will resolve to “No”.\n\nThe resolution source for this market will be a consensus of official Democratic Party sources.\n\nAny replacement of the democratic nominee before election day will not change the resolution of the market.", "commentCount": 616, "creationDate": "2025-07-11T18:41:17.827389Z", "electionType": "Democratic Nomination", "gmpChartMode": "default", "openInterest": 11026102.525969, "enableNegRisk": true, "estimateValue": false, "eventMetadata": {"context_updated_at": "2026-03-29T06:30:52.944Z", "context_description": "California Governor Gavin Newsom commands trader consensus at 24% implied probability for the 2028 Democratic presidential nomination, driven by his March 12 home-state poll lead over Kamala Harris by 14 points, ongoing book tours in early primary states like New Hampshire, and positioning as a national fundraiser post-2024 defeat. Alexandria Ocasio-Cortez trails at 8% on progressive grassroots appeal and recent international profiles like Munich appearances, while Jon Ossoff's 6% reflects Georgia swing-state incumbency. This wide-open field diverges from mixed national polls—JL Partners (March 18-20) shows Harris at 22% over Newsom's 19%—highlighting market emphasis on executive experience versus polling. Consolidation could hinge on 2026 midterm results elevating battleground performers like Josh Shapiro or Gretchen Whitmer, early fundraising disclosures, and party endorsements ahead of Iowa caucuses.", "context_requires_regen": true}, "featuredOrder": 15, "liquidityClob": 43770146.56328, "enableOrderBook": true, "negRiskMarketID": "0x2c3d7e0eee6f058be3006baabf0d54a07da254ba47fe6e3e095e7990c7814700", "showAllOutcomes": true, "negRiskAugmented": true, "resolutionSource": "", "showMarketImages": true, "cumulativeMarkets": false, "pendingDeployment": false, "deployingTimestamp": "2025-07-11T18:14:44.108448Z", "automaticallyActive": true, "requiresTranslation": false}], "funded": false, "spread": 0.001, "volume": "24231964.76713505", "bestAsk": 0.006, "bestBid": 0.005, "endDate": "2028-11-07T00:00:00Z", "feeType": null, "negRisk": true, "umaBond": "25000", "approved": true, "archived": false, "featured": false, "outcomes": "[\"Yes\", \"No\"]", "question": "Will Raphael Warnock win the 2028 Democratic presidential nomination?", "createdAt": "2025-07-03T20:37:08.125174Z", "deploying": false, "liquidity": "1596308.44339", "startDate": "2025-07-11T18:36:11.106Z", "umaReward": "10", "updatedAt": "2026-03-29T06:43:14.795209Z", "volume1mo": 6280163.686772391, "volume1wk": 1574246.477223908, "volume1yr": 24231964.767131317, "volumeNum": 24231964.76713505, "endDateIso": "2028-11-07", "questionID": "0x2c3d7e0eee6f058be3006baabf0d54a07da254ba47fe6e3e095e7990c781470c", "resolvedBy": "0x2F5e3684cb1F318ec51b00Edba38d79Ac2c0aA9d", "restricted": true, "rfqEnabled": false, "volume24hr": 203979.83558099996, "volumeClob": 24231964.76713505, "competitive": 0.8035160254240507, "conditionId": "0xdce84960dce38aa4a5800a5eba7c9ac34d2ce49ba9d44c42572c472d468af264", "description": "This market will resolve to “Yes” if the named individual wins and accepts the 2028 nomination of the Democratic Party for U.S. president. Otherwise, this market will resolve to “No”.\n\nThe resolution source for this market will be a consensus of official Democratic Party sources.\n\nAny replacement of the democratic nominee before election day will not change the resolution of the market.", "feesEnabled": false, "seriesColor": "", "clobTokenIds": "[\"52310257194926233099477326083312959938983447523839326865869372741334281264830\", \"88403451835230950222119400360490338078378790763472355557584611572247419676051\"]", "liquidityNum": 1596308.44339, "negRiskOther": false, "orderMinSize": 5, "startDateIso": "2025-07-11", "submitted_by": "0x91430CaD2d3975766499717fA0D66A78D814E5c5", "liquidityClob": 1596308.44339, "outcomePrices": "[\"0.0055\", \"0.9945\"]", "showGmpSeries": false, "volume1moClob": 6280163.686772391, "volume1wkClob": 1574246.477223908, "volume1yrClob": 24231964.767131317, "customLiveness": 0, "groupItemTitle": "Raphael Warnock", "lastTradePrice": 0.005, "rewardsMinSize": 20, "showGmpOutcome": false, "volume24hrClob": 203979.83558099996, "acceptingOrders": true, "enableOrderBook": true, "negRiskMarketID": "0x2c3d7e0eee6f058be3006baabf0d54a07da254ba47fe6e3e095e7990c7814700", "clearBookOnStart": true, "hasReviewedDates": true, "manualActivation": false, "negRiskRequestID": "0x7582e1feb071a286ac4803ff6555fe830cded5480ede75b13f5de7325842e4e8", "resolutionSource": "", "rewardsMaxSpread": 3.5, "pendingDeployment": false, "deployingTimestamp": "2025-07-11T18:15:13.626487Z", "groupItemThreshold": "12", "marketMakerAddress": "", "oneWeekPriceChange": 0.001, "automaticallyActive": true, "oneMonthPriceChange": 0.003, "requiresTranslation": false, "holdingRewardsEnabled": true, "orderPriceMinTickSize": 0.001, "umaResolutionStatuses": "[]", "acceptingOrdersTimestamp": "2025-07-11T18:35:48Z", "pagerDutyNotificationEnabled": false}</t>
         </is>
       </c>
       <c r="AJ5" s="1" t="n">
-        <v>46110.0765398214</v>
+        <v>46110.28125473107</v>
       </c>
       <c r="AK5" s="1" t="n">
-        <v>46110.07659220583</v>
+        <v>46110.28125473107</v>
       </c>
     </row>
     <row r="6">
@@ -1172,7 +1172,7 @@
         <v>45841.85914017702</v>
       </c>
       <c r="L6" s="1" t="n">
-        <v>46110.07594215713</v>
+        <v>46110.28010830501</v>
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" s="2" t="n">
@@ -1212,22 +1212,22 @@
         <v>0.001</v>
       </c>
       <c r="Z6" t="n">
-        <v>36363010.82116401</v>
+        <v>36378433.74515404</v>
       </c>
       <c r="AA6" t="n">
-        <v>36363010.82116401</v>
+        <v>36378433.74515404</v>
       </c>
       <c r="AB6" t="n">
-        <v>1391311.375341021</v>
+        <v>1384211.555332022</v>
       </c>
       <c r="AC6" t="n">
-        <v>9684167.600489439</v>
+        <v>9658386.735839438</v>
       </c>
       <c r="AD6" t="n">
-        <v>36363010.82115652</v>
+        <v>36378433.74514653</v>
       </c>
       <c r="AE6" t="n">
-        <v>2072257.52847</v>
+        <v>2063705.89771</v>
       </c>
       <c r="AF6" t="inlineStr">
         <is>
@@ -1246,14 +1246,14 @@
       </c>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>{"id": "559666", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/will-tim-walz-win-the-2028-us-presidential-election-V8-ATYdzVQA9.png", "slug": "will-tim-walz-win-the-2028-democratic-presidential-nomination-475", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/will-tim-walz-win-the-2028-us-presidential-election-V8-ATYdzVQA9.png", "ready": false, "active": true, "closed": false, "events": [{"id": "30829", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/democrats+2028+donkey.png", "slug": "democratic-presidential-nominee-2028", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/democrats+2028+donkey.png", "title": "Democratic Presidential Nominee 2028", "active": true, "closed": false, "sortBy": "price", "ticker": "democratic-presidential-nominee-2028", "volume": 929408692.9919622, "endDate": "2028-11-07T00:00:00Z", "negRisk": true, "archived": false, "featured": true, "createdAt": "2025-07-03T20:36:57.824243Z", "deploying": false, "liquidity": 44060833.8747, "startDate": "2025-07-11T18:41:17.827458Z", "startTime": "2028-11-07T12:00:00Z", "updatedAt": "2026-03-29T01:49:40.20413Z", "volume1mo": 201497523.6404877, "volume1wk": 53094243.130744666, "volume1yr": 929408692.9919566, "restricted": true, "volume24hr": 4958628.24913, "competitive": 0.9382691608050256, "countryName": "U.S.", "description": "This market will resolve to “Yes” if the named individual wins and accepts the 2028 nomination of the Democratic Party for U.S. president. Otherwise, this market will resolve to “No”.\n\nThe resolution source for this market will be a consensus of official Democratic Party sources.\n\nAny replacement of the democratic nominee before election day will not change the resolution of the market.", "commentCount": 616, "creationDate": "2025-07-11T18:41:17.827389Z", "electionType": "Democratic Nomination", "gmpChartMode": "default", "openInterest": 10925893.814415, "enableNegRisk": true, "estimateValue": false, "eventMetadata": {"context_updated_at": "2026-03-29T01:46:24.319Z", "context_description": "California Governor Gavin Newsom leads Polymarket's Democratic presidential nominee 2028 odds at 24.3% implied probability, driven by his March book tour in New Hampshire—testing early primary waters—and a March 12 California poll showing a 14-point edge over Kamala Harris, bolstering his executive experience and national anti-Trump profile amid party reckoning post-2024. Rep. Alexandria Ocasio-Cortez holds 8.3% on progressive grassroots energy and social media reach, though centrist groups like Third Way mobilized in March against left-wing frontrunners to prioritize electability. Sen. Jon Ossoff's 5.8% stems from Georgia battleground wins appealing to swing-state math. This fragmented field, with no outcome above 25%, could consolidate via 2026 midterm performances, fundraising dominance, key endorsements, or polling shifts favoring incumbents or moderates.", "context_requires_regen": true}, "featuredOrder": 15, "liquidityClob": 44060833.8747, "enableOrderBook": true, "negRiskMarketID": "0x2c3d7e0eee6f058be3006baabf0d54a07da254ba47fe6e3e095e7990c7814700", "showAllOutcomes": true, "negRiskAugmented": true, "resolutionSource": "", "showMarketImages": true, "cumulativeMarkets": false, "pendingDeployment": false, "deployingTimestamp": "2025-07-11T18:14:44.108448Z", "automaticallyActive": true, "requiresTranslation": false}], "funded": false, "spread": 0.001, "volume": "36363010.82116401", "bestAsk": 0.007, "bestBid": 0.006, "endDate": "2028-11-07T00:00:00Z", "feeType": null, "negRisk": true, "umaBond": "25000", "approved": true, "archived": false, "featured": false, "outcomes": "[\"Yes\", \"No\"]", "question": "Will Tim Walz win the 2028 Democratic presidential nomination?", "createdAt": "2025-07-03T20:37:09.711295Z", "deploying": false, "liquidity": "2072257.52847", "startDate": "2025-07-11T18:36:13.472Z", "umaReward": "10", "updatedAt": "2026-03-29T01:49:21.402376Z", "volume1mo": 9684167.60048944, "volume1wk": 1391311.3753410215, "volume1yr": 36363010.82115652, "volumeNum": 36363010.82116401, "endDateIso": "2028-11-07", "questionID": "0x2c3d7e0eee6f058be3006baabf0d54a07da254ba47fe6e3e095e7990c781470e", "resolvedBy": "0x2F5e3684cb1F318ec51b00Edba38d79Ac2c0aA9d", "restricted": true, "rfqEnabled": false, "volume24hr": 166373.48425700003, "volumeClob": 36363010.82116401, "competitive": 0.8041544225779221, "conditionId": "0x3265b10daeb30dbcc3214bd02e488551d0a5d3028392f4152e4750b943fbfc91", "description": "This market will resolve to “Yes” if the named individual wins and accepts the 2028 nomination of the Democratic Party for U.S. president. Otherwise, this market will resolve to “No”.\n\nThe resolution source for this market will be a consensus of official Democratic Party sources.\n\nAny replacement of the democratic nominee before election day will not change the resolution of the market.", "feesEnabled": false, "seriesColor": "", "clobTokenIds": "[\"104464678880204778606895232389511543522030897731392516718349574106843434770446\", \"90935594925886073322524509252821043048115343298080885997215308777385571383769\"]", "liquidityNum": 2072257.52847, "negRiskOther": false, "orderMinSize": 5, "startDateIso": "2025-07-11", "submitted_by": "0x91430CaD2d3975766499717fA0D66A78D814E5c5", "liquidityClob": 2072257.52847, "outcomePrices": "[\"0.0065\", \"0.9935\"]", "showGmpSeries": false, "volume1moClob": 9684167.60048944, "volume1wkClob": 1391311.3753410215, "volume1yrClob": 36363010.82115652, "customLiveness": 0, "groupItemTitle": "Tim Walz", "lastTradePrice": 0.007, "rewardsMinSize": 20, "showGmpOutcome": false, "volume24hrClob": 166373.48425700003, "acceptingOrders": true, "enableOrderBook": true, "negRiskMarketID": "0x2c3d7e0eee6f058be3006baabf0d54a07da254ba47fe6e3e095e7990c7814700", "clearBookOnStart": true, "hasReviewedDates": true, "manualActivation": false, "negRiskRequestID": "0x38954925500caffdcb0e0806f4f26109aec792bd3b4801975ec91830f3dac88c", "resolutionSource": "", "rewardsMaxSpread": 3.5, "oneDayPriceChange": 0.001, "pendingDeployment": false, "deployingTimestamp": "2025-07-11T18:15:13.74818Z", "groupItemThreshold": "14", "marketMakerAddress": "", "automaticallyActive": true, "oneMonthPriceChange": 0.003, "requiresTranslation": false, "holdingRewardsEnabled": true, "orderPriceMinTickSize": 0.001, "umaResolutionStatuses": "[]", "acceptingOrdersTimestamp": "2025-07-11T18:35:52Z", "pagerDutyNotificationEnabled": false}</t>
+          <t>{"id": "559666", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/will-tim-walz-win-the-2028-us-presidential-election-V8-ATYdzVQA9.png", "slug": "will-tim-walz-win-the-2028-democratic-presidential-nomination-475", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/will-tim-walz-win-the-2028-us-presidential-election-V8-ATYdzVQA9.png", "ready": false, "active": true, "closed": false, "events": [{"id": "30829", "new": false, "cyom": false, "icon": "https://polymarket-upload.s3.us-east-2.amazonaws.com/democrats+2028+donkey.png", "slug": "democratic-presidential-nominee-2028", "image": "https://polymarket-upload.s3.us-east-2.amazonaws.com/democrats+2028+donkey.png", "title": "Democratic Presidential Nominee 2028", "active": true, "closed": false, "sortBy": "price", "ticker": "democratic-presidential-nominee-2028", "volume": 930647837.2445823, "endDate": "2028-11-07T00:00:00Z", "negRisk": true, "archived": false, "featured": true, "createdAt": "2025-07-03T20:36:57.824243Z", "deploying": false, "liquidity": 43770146.56328, "startDate": "2025-07-11T18:41:17.827458Z", "startTime": "2028-11-07T12:00:00Z", "updatedAt": "2026-03-29T06:44:46.607657Z", "volume1mo": 201648772.32079622, "volume1wk": 51178107.61075467, "volume1yr": 930647837.2445767, "restricted": true, "volume24hr": 5365195.267472, "competitive": 0.9382691608050256, "countryName": "U.S.", "description": "This market will resolve to “Yes” if the named individual wins and accepts the 2028 nomination of the Democratic Party for U.S. president. Otherwise, this market will resolve to “No”.\n\nThe resolution source for this market will be a consensus of official Democratic Party sources.\n\nAny replacement of the democratic nominee before election day will not change the resolution of the market.", "commentCount": 616, "creationDate": "2025-07-11T18:41:17.827389Z", "electionType": "Democratic Nomination", "gmpChartMode": "default", "openInterest": 11026102.525969, "enableNegRisk": true, "estimateValue": false, "eventMetadata": {"context_updated_at": "2026-03-29T06:30:52.944Z", "context_description": "California Governor Gavin Newsom commands trader consensus at 24% implied probability for the 2028 Democratic presidential nomination, driven by his March 12 home-state poll lead over Kamala Harris by 14 points, ongoing book tours in early primary states like New Hampshire, and positioning as a national fundraiser post-2024 defeat. Alexandria Ocasio-Cortez trails at 8% on progressive grassroots appeal and recent international profiles like Munich appearances, while Jon Ossoff's 6% reflects Georgia swing-state incumbency. This wide-open field diverges from mixed national polls—JL Partners (March 18-20) shows Harris at 22% over Newsom's 19%—highlighting market emphasis on executive experience versus polling. Consolidation could hinge on 2026 midterm results elevating battleground performers like Josh Shapiro or Gretchen Whitmer, early fundraising disclosures, and party endorsements ahead of Iowa caucuses.", "context_requires_regen": true}, "featuredOrder": 15, "liquidityClob": 43770146.56328, "enableOrderBook": true, "negRiskMarketID": "0x2c3d7e0eee6f058be3006baabf0d54a07da254ba47fe6e3e095e7990c7814700", "showAllOutcomes": true, "negRiskAugmented": true, "resolutionSource": "", "showMarketImages": true, "cumulativeMarkets": false, "pendingDeployment": false, "deployingTimestamp": "2025-07-11T18:14:44.108448Z", "automaticallyActive": true, "requiresTranslation": false}], "funded": false, "spread": 0.001, "volume": "36378433.74515404", "bestAsk": 0.007, "bestBid": 0.006, "endDate": "2028-11-07T00:00:00Z", "feeType": null, "negRisk": true, "umaBond": "25000", "approved": true, "archived": false, "featured": false, "outcomes": "[\"Yes\", \"No\"]", "question": "Will Tim Walz win the 2028 Democratic presidential nomination?", "createdAt": "2025-07-03T20:37:09.711295Z", "deploying": false, "liquidity": "2063705.89771", "startDate": "2025-07-11T18:36:13.472Z", "umaReward": "10", "updatedAt": "2026-03-29T06:43:21.357553Z", "volume1mo": 9658386.735839438, "volume1wk": 1384211.5553320218, "volume1yr": 36378433.74514653, "volumeNum": 36378433.74515404, "endDateIso": "2028-11-07", "questionID": "0x2c3d7e0eee6f058be3006baabf0d54a07da254ba47fe6e3e095e7990c781470e", "resolvedBy": "0x2F5e3684cb1F318ec51b00Edba38d79Ac2c0aA9d", "restricted": true, "rfqEnabled": false, "volume24hr": 145337.90291499998, "volumeClob": 36378433.74515404, "competitive": 0.8041544225779221, "conditionId": "0x3265b10daeb30dbcc3214bd02e488551d0a5d3028392f4152e4750b943fbfc91", "description": "This market will resolve to “Yes” if the named individual wins and accepts the 2028 nomination of the Democratic Party for U.S. president. Otherwise, this market will resolve to “No”.\n\nThe resolution source for this market will be a consensus of official Democratic Party sources.\n\nAny replacement of the democratic nominee before election day will not change the resolution of the market.", "feesEnabled": false, "seriesColor": "", "clobTokenIds": "[\"104464678880204778606895232389511543522030897731392516718349574106843434770446\", \"90935594925886073322524509252821043048115343298080885997215308777385571383769\"]", "liquidityNum": 2063705.89771, "negRiskOther": false, "orderMinSize": 5, "startDateIso": "2025-07-11", "submitted_by": "0x91430CaD2d3975766499717fA0D66A78D814E5c5", "liquidityClob": 2063705.89771, "outcomePrices": "[\"0.0065\", \"0.9935\"]", "showGmpSeries": false, "volume1moClob": 9658386.735839438, "volume1wkClob": 1384211.5553320218, "volume1yrClob": 36378433.74514653, "customLiveness": 0, "groupItemTitle": "Tim Walz", "lastTradePrice": 0.007, "rewardsMinSize": 20, "showGmpOutcome": false, "volume24hrClob": 145337.90291499998, "acceptingOrders": true, "enableOrderBook": true, "negRiskMarketID": "0x2c3d7e0eee6f058be3006baabf0d54a07da254ba47fe6e3e095e7990c7814700", "clearBookOnStart": true, "hasReviewedDates": true, "manualActivation": false, "negRiskRequestID": "0x38954925500caffdcb0e0806f4f26109aec792bd3b4801975ec91830f3dac88c", "resolutionSource": "", "rewardsMaxSpread": 3.5, "oneDayPriceChange": 0.001, "pendingDeployment": false, "deployingTimestamp": "2025-07-11T18:15:13.74818Z", "groupItemThreshold": "14", "marketMakerAddress": "", "automaticallyActive": true, "oneMonthPriceChange": 0.003, "requiresTranslation": false, "holdingRewardsEnabled": true, "orderPriceMinTickSize": 0.001, "umaResolutionStatuses": "[]", "acceptingOrdersTimestamp": "2025-07-11T18:35:52Z", "pagerDutyNotificationEnabled": false}</t>
         </is>
       </c>
       <c r="AJ6" s="1" t="n">
-        <v>46110.0765398214</v>
+        <v>46110.28125473107</v>
       </c>
       <c r="AK6" s="1" t="n">
-        <v>46110.07659220583</v>
+        <v>46110.28125473107</v>
       </c>
     </row>
   </sheetData>
@@ -1267,7 +1267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1304,122 +1304,26 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>553878</v>
+        <v>559666</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Will the Chicago Bulls win the 2026 NBA Finals? This market will resolve to “Yes” if the Chicago Bulls win the 2026 NBA Finals. Otherwise, this market will resolve to “No”. This market will resolve to “No” if it becomes impossible for this team to win the 2026 NBA Finals based off the rules of the NBA. The resolution source for this market will be information from the NBA.</t>
+          <t>k2_react_agent</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[{"url": "https://www.forecasterarena.com/markets/1765056787079-j5pq77xd8", "score": 0.9281033, "title": "AI Models Competing in Prediction Markets - Forecaster Arena", "content": "This market will resolve to “Yes” if the Chicago Bulls win the 2026 NBA Finals. Otherwise, this market will resolve to “No”. This market will resolve to “No", "raw_content": null}, {"url": "https://polysimulator.com/markets/0xf374fb58698bccedf29399f9f5548a70370a11c0fece34f2570fb9b3885e8e5a", "score": 0.92507464, "title": "Will the Chicago Bulls win the 2026 NBA Finals? - PolySimulator", "content": "Resolution Criteria. This market will resolve to “Yes” if the Chicago Bulls win the 2026 NBA Finals. Otherwise, this market will resolve to “No”.", "raw_content": null}, {"url": "https://www.frenflow.com/polymarket/market/will-the-chicago-bulls-win-the-2026-nba-finals", "score": 0.8684817, "title": "Will the Chicago Bulls win the 2026 NBA Finals? | Yes 0% - No 100%", "content": "What are the current odds for \"Will the Chicago Bulls win the 2026 NBA Finals?\"? Traders currently give this a 0% chance of Yes and 100% chance of No. Odds", "raw_content": null}, {"url": "https://polysimulator.com/markets/0x00ca3a4205ea548274f06891fd4b703160675842dd0120279ef5a40f1ddcfdaa", "score": 0.86632514, "title": "Will the Chicago Bulls win the NBA Eastern Conference Finals?", "content": "This market will resolve to “Yes ... Otherwise, this market will resolve to “No”. This market will resolve to “No” if it becomes impossible for this team", "raw_content": null}, {"url": "https://pam.polymarket.com/event/2026-nba-champion/will-the-cleveland-cavaliers-win-the-2026-nba-finals", "score": 0.7900289, "title": "2026 NBA Champion Predictions &amp; Odds | Polymarket", "content": "This market will resolve to “Yes” if the Cleveland Cavaliers win the 2026 NBA Finals. Otherwise, this market will resolve to “No”. This market will resolve", "raw_content": null}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="E2" t="n">
         <v>5</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>46110.07659265352</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="n">
-        <v>553882</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Will the Charlotte Hornets win the 2026 NBA Finals? This market will resolve to “Yes” if the Charlotte Hornets win the 2026 NBA Finals. Otherwise, this market will resolve to “No”. This market will resolve to “No” if it becomes impossible for this team to win the 2026 NBA Finals based off the rules of the NBA. The resolution source for this market will be information from the NBA.</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>[{"url": "http://www.almanac.ai/m/will-the-charlotte-hornets-win-the-2026-nba-finals", "score": 0.9464435, "title": "Will the Charlotte Hornets win the 2026 NBA Finals? — 0.9% Odds ...", "content": "# Will the Charlotte Hornets win the 2026 NBA Finals? This market will resolve to “Yes” if the Charlotte Hornets win the 2026 NBA Finals. This market will resolve to “No” if it becomes impossible for this team to win the 2026 NBA Finals based off the rules of the NBA. Yes· 0.009shares @ 3.1¢. Yes· 0.007shares @ 3.1¢. Will the Indiana Pacers win the 2026 NBA Finals? 0.0%$86.9MWill the Memphis Grizzlies win the 2026 NBA Finals? 0.1%$34.2MWill the Chicago Bulls win the 2026 NBA Finals? 0.1%$22.5MWill the Utah Jazz win the 2026 NBA Finals? 0.1%$19.2MWill the Washington Wizards win the 2026 NBA Finals? 0.0%$18.0MWill the Brooklyn Nets win the 2026 NBA Finals? 0.0%$17.7MWill Chelsea win the 2025–26 English Premier League? 0.1%$75.2MWill Leeds win the 2025–26 English Premier League? 0.0%$38.4MWill Tottenham win the 2025–26 English Premier League? 0.0%$30.3MWill Slavia Pragu win the 2025–26 Champions League? 0.0%$28.4MWill Olympiakos win the 2025–26 Champions League? 0.0%$21.4MWill Club Brugge win the 2025–26 Champions League?", "raw_content": null}, {"url": "https://polyguana.com/market/553882", "score": 0.94584644, "title": "Will the Charlotte Hornets win the 2026 NBA Finals? - Polyguana", "content": "Resolution criteria: This market will resolve to “Yes” if the Charlotte Hornets win the 2026 NBA Finals. This market will resolve to “No” if it becomes impossible for this team to win the 2026 NBA Finals based off the rules of the NBA. The resolution source for this market will be information from the NBA. Resolution still depends heavily on the market rules text because no standalone canonical source URL is pinned yet. This market will resolve to “No” if it becomes impossible for this team to win the 2026 NBA Finals based off the rules of the NBA. The resolution source for this market will be information from the NBA. This market will resolve to “No” if it becomes impossible for this team to win the 2026 NBA Finals based off the rules of the NBA. The resolution source for this market will be information from the NBA.", "raw_content": null}, {"url": "https://parletto.bet/markets/553882", "score": 0.923268, "title": "Will the Charlotte Hornets win the 2026 NBA Finals? - Parletto ...", "content": "This market will resolve to “Yes” if the Charlotte Hornets win the 2026 NBA Finals. Otherwise, this market will resolve to “No”. This market will resolve to “No", "raw_content": null}, {"url": "https://www.predictionhunt.com/odds/2026-nba-champions", "score": 0.846159, "title": "2026 NBA Champions | Live Odds Comparison - Prediction Hunt", "content": "Live prediction market odds for 2026 NBA Champions. When does the market for the 2026 NBA Champions close? 2026 NBA Champions is a prediction market event currently tracked across 3 platforms (Kalshi, Polymarket, Opinion). ## Market Rulebook: 2026 NBA Champions. If Oklahoma City win the 2026 Pro Basketball Finals, then the market resolves to Yes. This market will resolve to \"Yes\" if the specified team wins the 2026 NBA Finals. This market will resolve to \"No\" if it becomes impossible for this team to win the 2026 NBA Finals under NBA rules. The resolution source for this market will be official information from the NBA. This market will resolve to “Yes” if the Oklahoma City Thunder win the 2026 NBA Finals. This market will resolve to “No” if it becomes impossible for this team to win the 2026 NBA Finals based off the rules of the NBA. The resolution source for this market will be information from the NBA.", "raw_content": null}, {"url": "https://polymarket.com/event/nba-eastern-conference-champion", "score": 0.5335682, "title": "NBA Eastern Conference Champion Predictions &amp; Odds | Polymarket", "content": "This market will resolve to “Yes” if the Detroit Pistons win the 2024-2025 NBA Eastern Conference finals. Otherwise, this market will resolve to “No”.", "raw_content": null}]</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>5</v>
-      </c>
-      <c r="F3" s="1" t="n">
-        <v>46110.07659265352</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="n">
-        <v>558960</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Will Uzbekistan win the 2026 FIFA World Cup? This market will resolve according to the national team that wins the 2026 FIFA World Cup. If at any point it becomes impossible for this team to win the FIFA World Cup based on the rules of FIFA (e.g., they are eliminated in the knockout stage), this market will resolve immediately to “No”. If the 2026 FIFA World Cup is permanently canceled or has not…</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>[{"url": "https://www.squawka.com/en/outright-markets/uzbekistan-world-cup-2026-odds/", "score": 0.7653308, "title": "Uzbekistan to win World Cup 2026 odds", "content": "# Uzbekistan to win World Cup 2026 odds: Probability, path to final, tactics, stats and confirmed squad. Outright markets ## Carabao Cup 2025-26 outright odds: Man City win the first trophy of the season. Outright markets ## Croatia to win World Cup 2026 odds: Probability, path to final, tactics, stats and confirmed squad. Croatia to win World Cup 2026 odds: Probability, path to final, tactics, stats and confirmed squad. Outright markets ## Colombia to win World Cup 2026 odds: Probability, path to final, tactics, stats and confirmed squad. Outright markets ## Canada to win World Cup 2026 odds: Probability, path to final, tactics, stats and confirmed squad. Outright markets ## Cape Verde to win World Cup 2026 odds: Probability, path to final, tactics, stats and confirmed squad. Outright markets ## Brazil to win World Cup 2026 odds: Probability, path to final, tactics, stats and confirmed squad. Outright markets ## Belgium to win World Cup 2026 odds: Probability, path to final, tactics, stats and confirmed squad.", "raw_content": null}, {"url": "https://sports.betmgm.com/en/blog/world-cup/uzbekistan-world-cup-odds-chances-to-win-world-cup-bm25/", "score": 0.7598145, "title": "Uzbekistan World Cup Odds: Chances To Win 2026 World Cup", "content": "Has Uzbekistan Won the World Cup? No, Uzbekistan has never won the World Cup. They have yet to qualify for a World Cup tournament.", "raw_content": null}, {"url": "https://www.quora.com/What-is-the-likelihood-that-the-winner-of-the-FIFA-World-Cup-2026-be-one-of-the-host-nations-or-a-country-that-has-not-previously-won-it-Or-in-reality-if-Spain-implode-in-the-early-stages-are-the-usual-suspects", "score": 0.34072697, "title": "What is the likelihood that the winner of the FIFA World Cup ...", "content": "What is the likelihood that the winner of the FIFA World Cup 2026 be one of the host nations, or a country that has not previously won it?", "raw_content": null}]</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>46110.07659265352</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B5" t="n">
-        <v>559664</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Will Raphael Warnock win the 2028 Democratic presidential nomination? This market will resolve to “Yes” if the named individual wins and accepts the 2028 nomination of the Democratic Party for U.S. president. Otherwise, this market will resolve to “No”. The resolution source for this market will be a consensus of official Democratic Party sources. Any replacement of the democratic nominee before…</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>[{"url": "https://www.independent.co.uk/news/world/americas/us-politics/2028-election-democrats-nominee-raphael-warnock-b2890565.html", "score": 0.82048416, "title": "CNN panel identifies 2028 frontrunners for Democrats", "content": "## Senator Raphael Warnock of Georgia was named as a possible candidate to be the 2028 Democratic presidential nominee. A CNN panel has identified the Democratic frontrunners for the 2028 presidential election with a new name added to the mix. While there’s been talk about California Governor Gavin Newsom’s rise in popularity thanks to his social media trolling efforts against President Donald Trump and a potential matchup between progressive congresswoman Alexandria Ocasio-Cortez, also known as AOC, and Vice President JD Vance, there’s one Democrat some may be overlooking. A CNN panel has identified the Democratic frontrunners, such as California Governor Gavin Newsom, for the 2028 presidential election with a new name added to the mix. Bash said Newsom’s odds “shot up,” showing that he has a 36 percent chance at being the Democratic presidential nominee. Bloomberg opinion columnist Nia Malika Henderson said she would add Senator Raphael Warnock of Georgia to the list of potential 2028 Democratic presidential nominees.", "raw_content": null}, {"url": "https://www.govtrack.us/congress/members/raphael_warnock/456858", "score": 0.6862234, "title": "Sen. Raphael Warnock [D-GA, 2021-2028], Senator ...", "content": "Warnock is the junior senator from Georgia and is a Democrat. He has served since Jan 20, 2021. Warnock is next up for reelection in 2028 and serves until Jan", "raw_content": null}, {"url": "https://newrepublic.com/article/206361/transcript-democrats-best-positioned-win-2028-nomination", "score": 0.559411, "title": "The Democrats Best Positioned To Win the 2028 Nomination", "content": "**Conroy:** I think my pick is going to probably allow you to have the one that you wanted to go first anyway, since Nathaniel is second. At FiveThirtyEight, we used to have these conversations years ago about Gavin Newsom, and as the resident—other people worked at and lived in California, were from California at FiveThirtyEight—but I was like, “I just don’t think it’s going to happen.” But he does. **Bacon:** I don’t think Warnock wants to run, so I’m going to go with Ossoff. **Conroy:** I’ll quickly say: In the world I’m seeing, when the primaries happen again, I had suggested I think there is going to be a big backlash against the Trump administration. **Bacon.:** So I chose Ossoff because I think he’s going to win this Georgia Senate race. I don’t think he’s going to win the Black vote overwhelmingly, because I have no evidence of that. **Bacon:** No, I think Wes Moore *is* going to run. But I don’t think he’s going to run.", "raw_content": null}, {"url": "https://polymarket.com/event/democratic-presidential-nominee-2028", "score": 0.338493, "title": "Democratic Presidential Nominee 2028 Predictions &amp; Odds", "content": "# Democratic Presidential Nominee 2028. # Democratic Presidential Nominee 2028. Gavin Newsom leads trader consensus at 24.3% implied probability for the 2028 Democratic presidential nomination in a wide-open field following Kamala Harris's 2024 general election loss, driven by his executive experience as California governor, robust national fundraising exceeding $50 million post-election, and high-profile anti-Trump positioning through media appearances and early primary-state visits. Gavin Newsom leads trader consensus at 24.3% implied probability for the 2028 Democratic presidential nomination in a wide-open field following Kamala Harris's 2024 general election loss, driven by his executive experience as California governor, robust national fundraising exceeding $50 million post-election, and high-profile anti-Trump positioning through media appearances and early primary-state visits. ### What is the \"Democratic Presidential Nominee 2028\" prediction market? ### How much trading activity has \"Democratic Presidential Nominee 2028\" generated on Polymarket? ### How do I trade on \"Democratic Presidential Nominee 2028\"? ### When does the \"Democratic Presidential Nominee 2028\" market close?", "raw_content": null}, {"url": "https://www.270towin.com/2028-democratic-nomination/", "score": 0.2830381, "title": "2028 Democratic Presidential Nomination", "content": "| | [Echelon Insights](https://echelonin.wpenginepowered.com/wp-content/uploads/August-2025-Voter-Omnibus-Topline-External.pdf) | 8/18/2025 | 522 LV | 26% | 13% | 6% | 11% | 3% | 3% | - | 5% | 2% | 3% | 2% | - | 0% | 1% | - | 3% | 2% | 0% | 0% | 0% | - | - | 0% | 0% | - | 1% | 1% | - | 18% |. | | [Echelon Insights](https://echelonin.wpenginepowered.com/wp-content/uploads/May-2025-Voter-Omnibus-Topline-External.pdf) | 5/12/2025 | 471 LV | 32% | 5% | 8% | 10% | 2% | 5% | - | 6% | 5% | 2% | 1% | - | 1% | 1% | - | 3% | 2% | - | 1% | 0% | - | - | 1% | 1% | - | 0% | 1% | - | 13% |.", "raw_content": null}]</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F5" s="1" t="n">
-        <v>46110.07659265352</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" t="n">
-        <v>559666</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Will Tim Walz win the 2028 Democratic presidential nomination? This market will resolve to “Yes” if the named individual wins and accepts the 2028 nomination of the Democratic Party for U.S. president. Otherwise, this market will resolve to “No”. The resolution source for this market will be a consensus of official Democratic Party sources. Any replacement of the democratic nominee before electio…</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>[{"url": "https://cryptorank.io/prediction-markets/democratic-presidential-nominee-2028", "score": 0.71185225, "title": "Democratic Presidential Nominee 2028 - CryptoRank.io", "content": "Will Jon Ossoff win the 2028 Democratic presidential nomination? Will Josh Shapiro win the 2028 Democratic presidential nomination? Will James Talarico win the 2028 Democratic presidential nomination? Will Jon Stewart win the 2028 Democratic presidential nomination? Will Andy Beshear win the 2028 Democratic presidential nomination? Will Mark Kelly win the 2028 Democratic presidential nomination? Will Ro Khanna win the 2028 Democratic presidential nomination? Will Wes Moore win the 2028 Democratic presidential nomination? Will Michelle Obama win the 2028 Democratic presidential nomination? Will Chris Murphy win the 2028 Democratic presidential nomination? Will Mark Cuban win the 2028 Democratic presidential nomination? Smith win the 2028 Democratic presidential nomination? Will LeBron James win the 2028 Democratic presidential nomination? Will MrBeast win the 2028 Democratic presidential nomination? Will Hillary Clinton win the 2028 Democratic presidential nomination? Will Chelsea Clinton win the 2028 Democratic presidential nomination? Will Phil Murphy win the 2028 Democratic presidential nomination? Will Barack Obama win the 2028 Democratic presidential nomination?", "raw_content": null}, {"url": "https://www.congress.gov/event/119th-congress/house-event/LC74924/text", "score": 0.20008872, "title": "A HEARING WITH SANCTUARY STATE GOVERNORS", "content": "Yes or no, Governor Walz? Governor Walz. If due process is given, certainly. Mr. Palmer. Governor Pritzker? Governor Pritzker. Exactly. We need due process", "raw_content": null}, {"url": "https://www.reddit.com/r/Askpolitics/comments/1ja1f9t/are_democrats_ok_with_the_party_doing_nothing/", "score": 0.10793502, "title": "Are Democrats ok with the party doing nothing under the guise of an ...", "content": "No, no they do not! Not only did every Democratic Senator and Bernie vote to confirm Rubio, we also had Democrats voting for Noem and Duffy and", "raw_content": null}, {"url": "https://www.facebook.com/mikethompsonforcongress/posts/excited-to-file-for-reelection-my-top-priority-is-fighting-for-our-democracy-and/1309681064305913/", "score": 0.043989986, "title": "Excited to file for reelection! My top priority is fighting for our ...", "content": "In this country, if there is no clear front running Democrat in a Congressional District, Congressman Steve Israel and the Democratic", "raw_content": null}, {"url": "https://www.facebook.com/KSTPTV/posts/a-tale-of-two-budgets-minnesota-is-projected-to-have-a-25-billion-surplus-going-/1266122748880170/", "score": 0.028438793, "title": "A tale of two budgets: Minnesota is projected to have a $2.5 billion ...", "content": "I am stating what our surpluses were in past years and yes projected amount for this year, which is almost over. ... No reasonable person could", "raw_content": null}]</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>5</v>
-      </c>
-      <c r="F6" s="1" t="n">
-        <v>46110.07659265352</v>
+        <v>46110.28129429565</v>
       </c>
     </row>
   </sheetData>
@@ -1433,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1475,266 +1379,32 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>553878</v>
+        <v>559666</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>## Investment Thesis: Chicago Bulls 2026 NBA Finals
-**1. Probability Estimate:** 1%
-**2. Key Supporting Evidence:**
-*   **Overwhelming Market Consensus:** The most direct market data (Frenflow, Source 3) indicates a 0% chance of the Bulls winning the 2026 NBA Finals, reflecting a strong consensus among traders that this outcome is highly improbable.
-*   **Current Team Performance &amp; Outlook:** The Chicago Bulls are not currently considered an NBA championship contender. They have not been a top-tier team for many years and lack the superstar talent and roster depth typically required to win an NBA title.
-*   **Long-Term Odds:** Winning an NBA Finals requires a sustained period of elite performance, a deep and cohesive roster, and often multiple superstar-level players. For a team currently outside the top tier, achieving this within two seasons (by 2026) would necessitate an extraordinary and unlikely series of events (e.g., multiple blockbuster trades, a generational draft pick, or unprecedented player development).
-**3. Key Risks / Counter-Arguments:**
-*   **Unforeseen Roster Overhaul:** The Bulls could execute multiple highly successful trades, draft a future superstar, or sign significant free agents that dramatically transform their roster and competitiveness.
-*   **Rapid Player Development:** Existing young players could develop into All-NBA talents faster than anticipated, forming a core capable of contending.
-*   **Market Inefficiency (Low Probability):** While the 0% market consensus is strong, there's always a minuscule chance of a black swan event or a significant market mispricing for an event two years in the future.
-*   **Injuries/Underperformance of Top Teams:** A significant decline or injury crisis among several top contenders could theoretically open a narrow window for a less-favored team.
-**4. Recommended Position:** **NO**</t>
+          <t>FN_CALL=True
+tavily_search(query="Tim Walz 2028 Democratic presidential nomination prospects", search_depth="advanced", time_range="year", topic="news")</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">### 1. AI Models Competing in Prediction Markets - Forecaster Arena
-URL: https://www.forecasterarena.com/markets/1765056787079-j5pq77xd8
-This market will resolve to “Yes” if the Chicago Bulls win the 2026 NBA Finals. Otherwise, this market will resolve to “No”. This market will resolve to “No
-### 2. Will the Chicago Bulls win the 2026 NBA Finals? - PolySimulator
-URL: https://polysimulator.com/markets/0xf374fb58698bccedf29399f9f5548a70370a11c0fece34f2570fb9b3885e8e5a
-Resolution Criteria. This market will resolve to “Yes” if the Chicago Bulls win the 2026 NBA Finals. Otherwise, this market will resolve to “No”.
-### 3. Will the Chicago Bulls win the 2026 NBA Finals? | Yes 0% - No 100%
-URL: https://www.frenflow.com/polymarket/market/will-the-chicago-bulls-win-the-2026-nba-finals
-What are the current odds for "Will the Chicago Bulls win the 2026 NBA Finals?"? Traders currently give this a 0% chance of Yes and 100% chance of No. Odds
-### 4. Will the Chicago Bulls win the NBA Eastern Conference Finals?
-URL: https://polysimulator.com/markets/0x00ca3a4205ea548274f06891fd4b703160675842dd0120279ef5a40f1ddcfdaa
-This market will resolve to “Yes ... Otherwise, this market will resolve to “No”. This market will resolve to “No” if it becomes impossible for this team
-### 5. 2026 NBA Champion Predictions &amp; Odds | Polymarket
-URL: https://pam.polymarket.com/event/2026-nba-champion/will-the-cleveland-cavaliers-win-the-2026-nba-finals
-This market will resolve to “Yes” if the Cleveland Cavaliers win the 2026 NBA Finals. Otherwise, this market will resolve to “No”. This market will resolve
-</t>
+          <t>{"agent_thinking_excerpt": "", "reasoning_steps": 3}</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>gemini-2.5-flash</t>
+          <t>MBZUAI-IFM/K2-Think-v2-ReAct</t>
         </is>
       </c>
       <c r="G2" s="1" t="n">
-        <v>46110.07659265352</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="n">
-        <v>553882</v>
-      </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>## Investment Thesis
-**1. Probability Estimate:** 1%
-**2. Key Supporting Evidence:**
-*   **Current Market Odds:** Prediction markets overwhelmingly assign a very low probability to the Charlotte Hornets winning the 2026 NBA Finals. Almanac.ai, for instance, lists their odds at just 0.9% (Source 1). This reflects the collective wisdom of market participants who do not see the Hornets as a contender.
-*   **Historical Performance &amp; Current Standing:** The Charlotte Hornets have never won an NBA championship and are not currently considered an elite team or a future contender based on their current roster and trajectory. Winning an NBA title requires a confluence of superstar talent, depth, coaching, and favorable circumstances, which the Hornets are far from possessing.
-*   **Short Timeline for Transformation:** To go from their current state to an NBA champion in just two seasons (by 2026) would require an unprecedented and rapid acquisition of multiple top-tier players, significant internal development, and a highly successful draft, which is an extremely low probability scenario.
-**3. Key Risks / Counter-arguments:**
-*   **Unforeseen Roster Changes:** A highly impactful trade for a superstar player or a significant free-agent signing, combined with exceptional draft picks, could theoretically accelerate their timeline.
-*   **Exceptional Player Development:** A rapid and unexpected leap in performance from their young core (e.g., LaMelo Ball, Brandon Miller) could make them more competitive than currently projected.
-*   **Market Inefficiency:** While unlikely for a major sports market, there's always a remote chance that current market odds are underestimating their true long-term potential.
-**4. Recommended Position:** NO</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">### 1. Will the Charlotte Hornets win the 2026 NBA Finals? — 0.9% Odds ...
-URL: http://www.almanac.ai/m/will-the-charlotte-hornets-win-the-2026-nba-finals
-# Will the Charlotte Hornets win the 2026 NBA Finals? This market will resolve to “Yes” if the Charlotte Hornets win the 2026 NBA Finals. This market will resolve to “No” if it becomes impossible for this team to win the 2026 NBA Finals based off the rules of the NBA. Yes· 0.009shares @ 3.1¢. Yes· 0.007shares @ 3.1¢. Will the Indiana Pacers win the 2026 NBA Finals? 0.0%$86.9MWill the Memphis Grizzlies win the 2026 NBA Finals? 0.1%$34.2MWill the Chicago Bulls win the 2026 NBA Finals? 0.1%$22.5MWill the Utah Jazz win the 2026 NBA Finals? 0.1%$19.2MWill the Washington Wizards win the 2026 NBA Finals? 0.0%$18.0MWill the Brooklyn Nets win the 2026 NBA Finals? 0.0%$17.7MWill Chelsea win the 2025–26 English Premier League? 0.1%$75.2MWill Leeds win the 2025–26 English Premier League? 0.0%$38.4MWill Tottenham win the 2025–26 English Premier League? 0.0%$30.3MWill Slavia Pragu win the 2025–26 Champions League? 0.0%$28.4MWill Olympiakos win the 2025–26 Champions League? 0.0%$21.4MWill Club Brugge win the 2025–26 Champions League?
-### 2. Will the Charlotte Hornets win the 2026 NBA Finals? - Polyguana
-URL: https://polyguana.com/market/553882
-Resolution criteria: This market will resolve to “Yes” if the Charlotte Hornets win the 2026 NBA Finals. This market will resolve to “No” if it becomes impossible for this team to win the 2026 NBA Finals based off the rules of the NBA. The resolution source for this market will be information from the NBA. Resolution still depends heavily on the market rules text because no standalone canonical source URL is pinned yet. This market will resolve to “No” if it becomes impossible for this team to win the 2026 NBA Finals based off the rules of the NBA. The resolution source for this market will be information from the NBA. This market will resolve to “No” if it becomes impossible for this team to win the 2026 NBA Finals based off the rules of the NBA. The resolution source for this market will be information from the NBA.
-### 3. Will the Charlotte Hornets win the 2026 NBA Finals? - Parletto ...
-URL: https://parletto.bet/markets/553882
-This market will resolve to “Yes” if the Charlotte Hornets win the 2026 NBA Finals. Otherwise, this market will resolve to “No”. This market will resolve to “No
-### 4. 2026 NBA Champions | Live Odds Comparison - Prediction Hunt
-URL: https://www.predictionhunt.com/odds/2026-nba-champions
-Live prediction market odds for 2026 NBA Champions. When does the market for the 2026 NBA Champions close? 2026 NBA Champions is a prediction market event currently tracked across 3 platforms (Kalshi, Polymarket, Opinion). ## Market Rulebook: 2026 NBA Champions. If Oklahoma City win the 2026 Pro Basketball Finals, then the market resolves to Yes. This market will resolve to "Yes" if the specified team wins the 2026 NBA Finals. This market will resolve to "No" if it becomes impossible for this team to win the 2026 NBA Finals under NBA rules. The resolution source for this market will be official information from the NBA. This market will resolve to “Yes” if the Oklahoma City Thunder win the 2026 NBA Finals. This market will resolve to “No” if it becomes impossible for this team to win the 2026 NBA Finals based off the rules of the NBA. The resolution source for this market will be information from the NBA.
-### 5. NBA Eastern Conference Champion Predictions &amp; Odds | Polymarket
-URL: https://polymarket.com/event/nba-eastern-conference-champion
-This market will resolve to “Yes” if the Detroit Pistons win the 2024-2025 NBA Eastern Conference finals. Otherwise, this market will resolve to “No”.
-</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>gemini-2.5-flash</t>
-        </is>
-      </c>
-      <c r="G3" s="1" t="n">
-        <v>46110.07659265352</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="n">
-        <v>558960</v>
-      </c>
-      <c r="C4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>## Investment Thesis: Uzbekistan to Win 2026 FIFA World Cup
-**1. Probability Estimate:** 0.01%
-**2. Key Supporting Evidence:**
-*   **No Prior World Cup Qualification:** Uzbekistan has never qualified for a FIFA World Cup tournament in its history (Source 2). This is a fundamental hurdle, as they must first qualify to even have a chance to win.
-*   **No World Cup Wins:** Consequently, Uzbekistan has never won the World Cup (Source 2).
-*   **Historical Precedent:** Winning the FIFA World Cup is an extremely rare feat, typically achieved by a select group of established footballing powerhouses. For a nation that has never even qualified, winning the tournament represents an astronomical leap in performance and capability.
-**3. Key Risks / Counter-arguments:**
-*   **Expanded Tournament Format:** The 2026 FIFA World Cup will feature an expanded format with 48 teams, which could theoretically make qualification slightly easier for nations like Uzbekistan and potentially increase the chances of a "dark horse" reaching later stages.
-*   **Unforeseen Development:** While highly improbable, a sudden and dramatic rise in the quality of Uzbek football, combined with an exceptional generation of talent and a favorable draw, could theoretically lead to an unprecedented upset.
-*   **Market Resolution Clause:** The market resolves to "No" immediately upon elimination, which is a strong bias against a "Yes" outcome for any team, especially a long shot.
-**4. Recommended Position:** **NO**</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">### 1. Uzbekistan to win World Cup 2026 odds
-URL: https://www.squawka.com/en/outright-markets/uzbekistan-world-cup-2026-odds/
-# Uzbekistan to win World Cup 2026 odds: Probability, path to final, tactics, stats and confirmed squad. Outright markets ## Carabao Cup 2025-26 outright odds: Man City win the first trophy of the season. Outright markets ## Croatia to win World Cup 2026 odds: Probability, path to final, tactics, stats and confirmed squad. Croatia to win World Cup 2026 odds: Probability, path to final, tactics, stats and confirmed squad. Outright markets ## Colombia to win World Cup 2026 odds: Probability, path to final, tactics, stats and confirmed squad. Outright markets ## Canada to win World Cup 2026 odds: Probability, path to final, tactics, stats and confirmed squad. Outright markets ## Cape Verde to win World Cup 2026 odds: Probability, path to final, tactics, stats and confirmed squad. Outright markets ## Brazil to win World Cup 2026 odds: Probability, path to final, tactics, stats and confirmed squad. Outright markets ## Belgium to win World Cup 2026 odds: Probability, path to final, tactics, stats and confirmed squad.
-### 2. Uzbekistan World Cup Odds: Chances To Win 2026 World Cup
-URL: https://sports.betmgm.com/en/blog/world-cup/uzbekistan-world-cup-odds-chances-to-win-world-cup-bm25/
-Has Uzbekistan Won the World Cup? No, Uzbekistan has never won the World Cup. They have yet to qualify for a World Cup tournament.
-### 3. What is the likelihood that the winner of the FIFA World Cup ...
-URL: https://www.quora.com/What-is-the-likelihood-that-the-winner-of-the-FIFA-World-Cup-2026-be-one-of-the-host-nations-or-a-country-that-has-not-previously-won-it-Or-in-reality-if-Spain-implode-in-the-early-stages-are-the-usual-suspects
-What is the likelihood that the winner of the FIFA World Cup 2026 be one of the host nations, or a country that has not previously won it?
-</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>gemini-2.5-flash</t>
-        </is>
-      </c>
-      <c r="G4" s="1" t="n">
-        <v>46110.07659265352</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B5" t="n">
-        <v>559664</v>
-      </c>
-      <c r="C5" t="n">
-        <v>5</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>## Investment Thesis: Raphael Warnock for 2028 Democratic Presidential Nomination
-**Probability Estimate:** 2%
-**Key Supporting Evidence:**
-1.  **Extremely Low Polling Support:** Hypothetical 2028 Democratic primary polls show Senator Warnock with minimal support, registering only 1-3% among likely voters (Source 5). This places him far behind other potential candidates like Gavin Newsom, Kamala Harris, and Gretchen Whitmer.
-2.  **Not a Frontrunner in Prediction Markets:** Major prediction markets for the 2028 Democratic nomination, such as Polymarket, do not list Warnock among the leading contenders. Gavin Newsom, for instance, leads with a 24.3% implied probability, while Warnock is not even mentioned in the summary of significant candidates (Source 4).
-3.  **Doubt About Presidential Ambition:** At least one political analyst has explicitly stated, "I don't think Warnock wants to run" for president (Source 3), suggesting a lack of personal desire or strategic intent to pursue the nomination.
-4.  **Senate Re-election Conflict:** Warnock's current Senate term expires in 2028, meaning he would be up for re-election in the same year as the presidential election. This presents a significant strategic hurdle, as he would likely have to choose between seeking the presidency and defending his Senate seat (Source 2).
-**Key Risks / Counter-arguments:**
-1.  **On the Radar of Some Analysts:** A CNN panel and a Bloomberg opinion columnist have identified Warnock as a "possible candidate" or a "new name" in the 2028 Democratic field (Source 1), indicating he has some level of national recognition and is considered by some as a potential contender.
-2.  **National Profile:** As a sitting U.S. Senator from a key swing state (Georgia), Warnock possesses a national platform and fundraising capabilities that could be leveraged for a presidential bid if he chose to pursue one.
-3.  **Dynamic Political Landscape:** The political environment can shift dramatically over four years. Current frontrunners may face unforeseen challenges, opening opportunities for less expected candidates.
-**Recommended Position:** NO</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">### 1. CNN panel identifies 2028 frontrunners for Democrats
-URL: https://www.independent.co.uk/news/world/americas/us-politics/2028-election-democrats-nominee-raphael-warnock-b2890565.html
-## Senator Raphael Warnock of Georgia was named as a possible candidate to be the 2028 Democratic presidential nominee. A CNN panel has identified the Democratic frontrunners for the 2028 presidential election with a new name added to the mix. While there’s been talk about California Governor Gavin Newsom’s rise in popularity thanks to his social media trolling efforts against President Donald Trump and a potential matchup between progressive congresswoman Alexandria Ocasio-Cortez, also known as AOC, and Vice President JD Vance, there’s one Democrat some may be overlooking. A CNN panel has identified the Democratic frontrunners, such as California Governor Gavin Newsom, for the 2028 presidential election with a new name added to the mix. Bash said Newsom’s odds “shot up,” showing that he has a 36 percent chance at being the Democratic presidential nominee. Bloomberg opinion columnist Nia Malika Henderson said she would add Senator Raphael Warnock of Georgia to the list of potential 2028 Democratic presidential nominees.
-### 2. Sen. Raphael Warnock [D-GA, 2021-2028], Senator ...
-URL: https://www.govtrack.us/congress/members/raphael_warnock/456858
-Warnock is the junior senator from Georgia and is a Democrat. He has served since Jan 20, 2021. Warnock is next up for reelection in 2028 and serves until Jan
-### 3. The Democrats Best Positioned To Win the 2028 Nomination
-URL: https://newrepublic.com/article/206361/transcript-democrats-best-positioned-win-2028-nomination
-**Conroy:** I think my pick is going to probably allow you to have the one that you wanted to go first anyway, since Nathaniel is second. At FiveThirtyEight, we used to have these conversations years ago about Gavin Newsom, and as the resident—other people worked at and lived in California, were from California at FiveThirtyEight—but I was like, “I just don’t think it’s going to happen.” But he does. **Bacon:** I don’t think Warnock wants to run, so I’m going to go with Ossoff. **Conroy:** I’ll quickly say: In the world I’m seeing, when the primaries happen again, I had suggested I think there is going to be a big backlash against the Trump administration. **Bacon.:** So I chose Ossoff because I think he’s going to win this Georgia Senate race. I don’t think he’s going to win the Black vote overwhelmingly, because I have no evidence of that. **Bacon:** No, I think Wes Moore *is* going to run. But I don’t think he’s going to run.
-### 4. Democratic Presidential Nominee 2028 Predictions &amp; Odds
-URL: https://polymarket.com/event/democratic-presidential-nominee-2028
-# Democratic Presidential Nominee 2028. # Democratic Presidential Nominee 2028. Gavin Newsom leads trader consensus at 24.3% implied probability for the 2028 Democratic presidential nomination in a wide-open field following Kamala Harris's 2024 general election loss, driven by his executive experience as California governor, robust national fundraising exceeding $50 million post-election, and high-profile anti-Trump positioning through media appearances and early primary-state visits. Gavin Newsom leads trader consensus at 24.3% implied probability for the 2028 Democratic presidential nomination in a wide-open field following Kamala Harris's 2024 general election loss, driven by his executive experience as California governor, robust national fundraising exceeding $50 million post-election, and high-profile anti-Trump positioning through media appearances and early primary-state visits. ### What is the "Democratic Presidential Nominee 2028" prediction market? ### How much trading activity has "Democratic Presidential Nominee 2028" generated on Polymarket? ### How do I trade on "Democratic Presidential Nominee 2028"? ### When does the "Democratic Presidential Nominee 2028" market close?
-### 5. 2028 Democratic Presidential Nomination
-URL: https://www.270towin.com/2028-democratic-nomination/
-| | [Echelon Insights](https://echelonin.wpenginepowered.com/wp-content/uploads/August-2025-Voter-Omnibus-Topline-External.pdf) | 8/18/2025 | 522 LV | 26% | 13% | 6% | 11% | 3% | 3% | - | 5% | 2% | 3% | 2% | - | 0% | 1% | - | 3% | 2% | 0% | 0% | 0% | - | - | 0% | 0% | - | 1% | 1% | - | 18% |. | | [Echelon Insights](https://echelonin.wpenginepowered.com/wp-content/uploads/May-2025-Voter-Omnibus-Topline-External.pdf) | 5/12/2025 | 471 LV | 32% | 5% | 8% | 10% | 2% | 5% | - | 6% | 5% | 2% | 1% | - | 1% | 1% | - | 3% | 2% | - | 1% | 0% | - | - | 1% | 1% | - | 0% | 1% | - | 13% |.
-</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>gemini-2.5-flash</t>
-        </is>
-      </c>
-      <c r="G5" s="1" t="n">
-        <v>46110.07659265352</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" t="n">
-        <v>559666</v>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>## Investment Thesis:
-**Probability Estimate:** 3%
-**Key Supporting Evidence:**
-1.  **Absence from 2028 Democratic Presidential Nominee Prediction Markets:** The most compelling evidence is Tim Walz's complete absence from the extensive list of individuals considered for the 2028 Democratic nomination on CryptoRank.io (Research 1). This indicates he is not currently on the radar of prediction market participants as a viable or even notable contender.
-2.  **Lack of National Campaign Indicators:** The provided research confirms Walz's role as Governor of Minnesota (Research 2, 5) and his participation in state-level political discussions. However, there is no evidence suggesting he is building a national profile, fundraising for a presidential bid, or generating significant national attention that would be prerequisite for a presidential nomination.
-**Key Risks / Counter-arguments:**
-1.  **Early Stage:** 2028 is still several years away, and political landscapes can shift dramatically. A candidate's profile and viability can change significantly over time.
-2.  **"Dark Horse" Potential:** While currently not a national figure, a sitting governor with a strong record (like Minnesota's budget surplus, Research 5) could theoretically emerge as a "dark horse" candidate, especially if other prominent figures decline to run or face unexpected challenges.
-**Recommended Position:** NO</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">### 1. Democratic Presidential Nominee 2028 - CryptoRank.io
-URL: https://cryptorank.io/prediction-markets/democratic-presidential-nominee-2028
-Will Jon Ossoff win the 2028 Democratic presidential nomination? Will Josh Shapiro win the 2028 Democratic presidential nomination? Will James Talarico win the 2028 Democratic presidential nomination? Will Jon Stewart win the 2028 Democratic presidential nomination? Will Andy Beshear win the 2028 Democratic presidential nomination? Will Mark Kelly win the 2028 Democratic presidential nomination? Will Ro Khanna win the 2028 Democratic presidential nomination? Will Wes Moore win the 2028 Democratic presidential nomination? Will Michelle Obama win the 2028 Democratic presidential nomination? Will Chris Murphy win the 2028 Democratic presidential nomination? Will Mark Cuban win the 2028 Democratic presidential nomination? Smith win the 2028 Democratic presidential nomination? Will LeBron James win the 2028 Democratic presidential nomination? Will MrBeast win the 2028 Democratic presidential nomination? Will Hillary Clinton win the 2028 Democratic presidential nomination? Will Chelsea Clinton win the 2028 Democratic presidential nomination? Will Phil Murphy win the 2028 Democratic presidential nomination? Will Barack Obama win the 2028 Democratic presidential nomination?
-### 2. A HEARING WITH SANCTUARY STATE GOVERNORS
-URL: https://www.congress.gov/event/119th-congress/house-event/LC74924/text
-Yes or no, Governor Walz? Governor Walz. If due process is given, certainly. Mr. Palmer. Governor Pritzker? Governor Pritzker. Exactly. We need due process
-### 3. Are Democrats ok with the party doing nothing under the guise of an ...
-URL: https://www.reddit.com/r/Askpolitics/comments/1ja1f9t/are_democrats_ok_with_the_party_doing_nothing/
-No, no they do not! Not only did every Democratic Senator and Bernie vote to confirm Rubio, we also had Democrats voting for Noem and Duffy and
-### 4. Excited to file for reelection! My top priority is fighting for our ...
-URL: https://www.facebook.com/mikethompsonforcongress/posts/excited-to-file-for-reelection-my-top-priority-is-fighting-for-our-democracy-and/1309681064305913/
-In this country, if there is no clear front running Democrat in a Congressional District, Congressman Steve Israel and the Democratic
-### 5. A tale of two budgets: Minnesota is projected to have a $2.5 billion ...
-URL: https://www.facebook.com/KSTPTV/posts/a-tale-of-two-budgets-minnesota-is-projected-to-have-a-25-billion-surplus-going-/1266122748880170/
-I am stating what our surpluses were in past years and yes projected amount for this year, which is almost over. ... No reasonable person could
-</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>gemini-2.5-flash</t>
-        </is>
-      </c>
-      <c r="G6" s="1" t="n">
-        <v>46110.07659265352</v>
+        <v>46110.28129429565</v>
       </c>
     </row>
   </sheetData>

</xml_diff>